<commit_message>
Updated the Portfolio Management Allocation Calculation Method
</commit_message>
<xml_diff>
--- a/financial_models/Stock_Monitor_CN.xlsx
+++ b/financial_models/Stock_Monitor_CN.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerry\PycharmProjects\Invest_Proc\financial_models\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kamanl/PycharmProjects/Invest_Proc/financial_models/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEA03B1A-B27B-455E-AB67-F4DF805F7CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E33AC718-416A-6348-BC7F-5345EDFFADC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-100" yWindow="-100" windowWidth="17120" windowHeight="10760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="投资组合管理" sheetId="10" r:id="rId1"/>
@@ -30,6 +30,19 @@
     <definedName name="WW3f877d8e32714ec8a8180854ed7f8276_634328482352282765" hidden="1">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -2168,7 +2181,7 @@
     <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2915,10 +2928,10 @@
     </xf>
   </cellXfs>
   <cellStyles count="4">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="3" xr:uid="{32ADA8AA-F280-4250-ABBF-7E6B9CB799DC}"/>
-    <cellStyle name="超链接" xfId="2" builtinId="8"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
@@ -2979,9 +2992,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3019,7 +3032,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3125,7 +3138,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3267,7 +3280,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3279,7 +3292,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E95"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.65"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="2.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="30" style="1" bestFit="1" customWidth="1"/>
@@ -3288,12 +3301,12 @@
     <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A1" s="20" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A2" s="21" t="s">
         <v>236</v>
       </c>
@@ -3302,7 +3315,7 @@
       <c r="D2" s="21"/>
       <c r="E2" s="21"/>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B4" s="116" t="s">
         <v>237</v>
       </c>
@@ -3310,7 +3323,7 @@
       <c r="D4" s="117"/>
       <c r="E4" s="117"/>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A6" s="20" t="s">
         <v>60</v>
       </c>
@@ -3319,7 +3332,7 @@
       </c>
       <c r="C6" s="49"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B7" s="116" t="s">
         <v>353</v>
       </c>
@@ -3327,12 +3340,12 @@
       <c r="D7" s="117"/>
       <c r="E7" s="117"/>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B9" s="23" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B10" s="1" t="s">
         <v>240</v>
       </c>
@@ -3341,7 +3354,7 @@
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B11" s="1" t="s">
         <v>241</v>
       </c>
@@ -3350,16 +3363,16 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B13" s="23" t="s">
         <v>242</v>
       </c>
       <c r="C13" s="4"/>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B14" s="1" t="s">
         <v>243</v>
       </c>
@@ -3367,7 +3380,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B15" s="1" t="s">
         <v>244</v>
       </c>
@@ -3375,7 +3388,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B16" s="1" t="s">
         <v>245</v>
       </c>
@@ -3383,27 +3396,27 @@
         <v>248</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B18" s="23" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B19" s="24" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B20" s="24" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B21" s="24" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A23" s="25" t="s">
         <v>61</v>
       </c>
@@ -3412,7 +3425,7 @@
       </c>
       <c r="C23" s="49"/>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A24" s="18"/>
       <c r="B24" s="116" t="s">
         <v>253</v>
@@ -3421,10 +3434,10 @@
       <c r="D24" s="117"/>
       <c r="E24" s="117"/>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A25" s="18"/>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A26" s="18"/>
       <c r="B26" s="43" t="s">
         <v>255</v>
@@ -3433,7 +3446,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B27" s="26" t="s">
         <v>257</v>
       </c>
@@ -3442,7 +3455,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B28" s="26" t="s">
         <v>258</v>
       </c>
@@ -3451,7 +3464,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A30" s="20" t="s">
         <v>62</v>
       </c>
@@ -3460,7 +3473,7 @@
       </c>
       <c r="C30" s="49"/>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A31" s="20"/>
       <c r="B31" s="43" t="s">
         <v>260</v>
@@ -3475,7 +3488,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="12" thickBot="1">
+    <row r="32" spans="1:5" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A32" s="20"/>
       <c r="B32" s="89" t="s">
         <v>263</v>
@@ -3492,7 +3505,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B33" s="92" t="s">
         <v>264</v>
       </c>
@@ -3508,7 +3521,7 @@
         <v>0.25000000000000006</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="12" thickBot="1">
+    <row r="34" spans="1:5" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B34" s="96" t="s">
         <v>265</v>
       </c>
@@ -3524,7 +3537,7 @@
         <v>9.0000000000000018</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B35" s="92" t="s">
         <v>266</v>
       </c>
@@ -3540,7 +3553,7 @@
         <v>0.12500000000000003</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="12" thickBot="1">
+    <row r="36" spans="1:5" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B36" s="96" t="s">
         <v>267</v>
       </c>
@@ -3556,7 +3569,7 @@
         <v>1.4999999999999998</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B37" s="100" t="s">
         <v>268</v>
       </c>
@@ -3572,15 +3585,15 @@
         <v>7.4999999999999997E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C38" s="86"/>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B39" s="20" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B40" s="117" t="s">
         <v>273</v>
       </c>
@@ -3588,7 +3601,7 @@
       <c r="D40" s="117"/>
       <c r="E40" s="117"/>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B41" s="116" t="s">
         <v>274</v>
       </c>
@@ -3596,7 +3609,7 @@
       <c r="D41" s="117"/>
       <c r="E41" s="117"/>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B42" s="116" t="s">
         <v>275</v>
       </c>
@@ -3604,7 +3617,7 @@
       <c r="D42" s="117"/>
       <c r="E42" s="117"/>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B43" s="116" t="s">
         <v>276</v>
       </c>
@@ -3612,7 +3625,7 @@
       <c r="D43" s="116"/>
       <c r="E43" s="116"/>
     </row>
-    <row r="44" spans="1:5" ht="34.35" customHeight="1">
+    <row r="44" spans="1:5" ht="34.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B44" s="117" t="s">
         <v>354</v>
       </c>
@@ -3620,7 +3633,7 @@
       <c r="D44" s="117"/>
       <c r="E44" s="117"/>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A46" s="21" t="s">
         <v>277</v>
       </c>
@@ -3629,7 +3642,7 @@
       <c r="D46" s="21"/>
       <c r="E46" s="21"/>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B48" s="117" t="s">
         <v>278</v>
       </c>
@@ -3637,12 +3650,12 @@
       <c r="D48" s="117"/>
       <c r="E48" s="117"/>
     </row>
-    <row r="50" spans="2:5">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B50" s="23" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="52" spans="2:5">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B52" s="43" t="s">
         <v>280</v>
       </c>
@@ -3652,7 +3665,7 @@
       <c r="D52" s="47"/>
       <c r="E52" s="47"/>
     </row>
-    <row r="53" spans="2:5">
+    <row r="53" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B53" s="26" t="s">
         <v>282</v>
       </c>
@@ -3663,7 +3676,7 @@
       <c r="D53" s="48"/>
       <c r="E53" s="46"/>
     </row>
-    <row r="54" spans="2:5">
+    <row r="54" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B54" s="26" t="s">
         <v>283</v>
       </c>
@@ -3674,7 +3687,7 @@
       <c r="D54" s="48"/>
       <c r="E54" s="46"/>
     </row>
-    <row r="55" spans="2:5">
+    <row r="55" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B55" s="26" t="s">
         <v>284</v>
       </c>
@@ -3687,12 +3700,12 @@
       </c>
       <c r="E55" s="46"/>
     </row>
-    <row r="57" spans="2:5">
+    <row r="57" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B57" s="23" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="59" spans="2:5">
+    <row r="59" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B59" s="43" t="s">
         <v>262</v>
       </c>
@@ -3706,7 +3719,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="60" spans="2:5">
+    <row r="60" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B60" s="26" t="s">
         <v>289</v>
       </c>
@@ -3721,7 +3734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="2:5">
+    <row r="61" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B61" s="26" t="s">
         <v>290</v>
       </c>
@@ -3736,7 +3749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="2:5">
+    <row r="62" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B62" s="26" t="s">
         <v>291</v>
       </c>
@@ -3751,7 +3764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="2:5">
+    <row r="63" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B63" s="26" t="s">
         <v>292</v>
       </c>
@@ -3766,7 +3779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="2:5">
+    <row r="64" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B64" s="26" t="s">
         <v>293</v>
       </c>
@@ -3781,7 +3794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.15">
       <c r="D65" s="27" t="s">
         <v>304</v>
       </c>
@@ -3790,7 +3803,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="12" thickBot="1">
+    <row r="66" spans="1:5" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="D66" s="41" t="s">
         <v>305</v>
       </c>
@@ -3799,23 +3812,23 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="12" thickTop="1"/>
-    <row r="68" spans="1:5">
+    <row r="67" spans="1:5" ht="13" thickTop="1" x14ac:dyDescent="0.15"/>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B68" s="1" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B69" s="1" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B70" s="1" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A72" s="21" t="s">
         <v>309</v>
       </c>
@@ -3824,7 +3837,7 @@
       <c r="D72" s="21"/>
       <c r="E72" s="21"/>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B74" s="117" t="s">
         <v>310</v>
       </c>
@@ -3832,7 +3845,7 @@
       <c r="D74" s="117"/>
       <c r="E74" s="117"/>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A76" s="28" t="s">
         <v>60</v>
       </c>
@@ -3840,12 +3853,12 @@
         <v>312</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B77" s="24" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A79" s="28" t="s">
         <v>200</v>
       </c>
@@ -3853,13 +3866,13 @@
         <v>313</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B80" s="1" t="str">
         <f>B19</f>
         <v>- 仅当ERB&gt;0且市场价格≤入场价格时具备配置资格</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B81" s="104" t="s">
         <v>314</v>
       </c>
@@ -3867,7 +3880,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B82" s="104" t="s">
         <v>315</v>
       </c>
@@ -3875,33 +3888,33 @@
         <v>191</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B83" s="103" t="str">
         <f>B20</f>
         <v xml:space="preserve">- 未入选标的获得正常配置额的50%	</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B85" s="20" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="86" spans="1:5">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B86" s="1" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B87" s="1" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="88" spans="1:5">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B88" s="1" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A90" s="21" t="s">
         <v>322</v>
       </c>
@@ -3910,22 +3923,22 @@
       <c r="D90" s="21"/>
       <c r="E90" s="21"/>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B92" s="20" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B93" s="24" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B94" s="24" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B95" s="24" t="s">
         <v>355</v>
       </c>
@@ -3954,7 +3967,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E95"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.65"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="2.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="30" style="1" bestFit="1" customWidth="1"/>
@@ -3963,12 +3976,12 @@
     <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A1" s="20" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A2" s="21" t="s">
         <v>51</v>
       </c>
@@ -3977,7 +3990,7 @@
       <c r="D2" s="21"/>
       <c r="E2" s="21"/>
     </row>
-    <row r="4" spans="1:5" ht="24.5" customHeight="1">
+    <row r="4" spans="1:5" ht="24.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B4" s="117" t="s">
         <v>149</v>
       </c>
@@ -3985,7 +3998,7 @@
       <c r="D4" s="117"/>
       <c r="E4" s="117"/>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A6" s="20" t="s">
         <v>60</v>
       </c>
@@ -3994,7 +4007,7 @@
       </c>
       <c r="C6" s="49"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B7" s="117" t="s">
         <v>201</v>
       </c>
@@ -4002,12 +4015,12 @@
       <c r="D7" s="117"/>
       <c r="E7" s="117"/>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B9" s="23" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B10" s="1" t="s">
         <v>58</v>
       </c>
@@ -4016,7 +4029,7 @@
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B11" s="1" t="s">
         <v>50</v>
       </c>
@@ -4025,16 +4038,16 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B13" s="23" t="s">
         <v>54</v>
       </c>
       <c r="C13" s="4"/>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B14" s="1" t="s">
         <v>145</v>
       </c>
@@ -4042,7 +4055,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B15" s="1" t="s">
         <v>133</v>
       </c>
@@ -4050,7 +4063,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B16" s="1" t="s">
         <v>134</v>
       </c>
@@ -4058,27 +4071,27 @@
         <v>132</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B18" s="23" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B19" s="24" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B20" s="24" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B21" s="24" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A23" s="25" t="s">
         <v>61</v>
       </c>
@@ -4087,7 +4100,7 @@
       </c>
       <c r="C23" s="49"/>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A24" s="18"/>
       <c r="B24" s="116" t="s">
         <v>203</v>
@@ -4096,10 +4109,10 @@
       <c r="D24" s="117"/>
       <c r="E24" s="117"/>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A25" s="18"/>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A26" s="18"/>
       <c r="B26" s="43" t="s">
         <v>135</v>
@@ -4108,7 +4121,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B27" s="26" t="s">
         <v>75</v>
       </c>
@@ -4116,7 +4129,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B28" s="26" t="s">
         <v>190</v>
       </c>
@@ -4124,7 +4137,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A30" s="20" t="s">
         <v>62</v>
       </c>
@@ -4133,7 +4146,7 @@
       </c>
       <c r="C30" s="49"/>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A31" s="20"/>
       <c r="B31" s="43" t="s">
         <v>204</v>
@@ -4148,7 +4161,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="12" thickBot="1">
+    <row r="32" spans="1:5" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A32" s="20"/>
       <c r="B32" s="89" t="s">
         <v>207</v>
@@ -4163,7 +4176,7 @@
         <v>-0.5</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B33" s="92" t="s">
         <v>210</v>
       </c>
@@ -4178,7 +4191,7 @@
         <v>0.25000000000000006</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="12" thickBot="1">
+    <row r="34" spans="1:5" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B34" s="96" t="s">
         <v>209</v>
       </c>
@@ -4194,7 +4207,7 @@
         <v>9.0000000000000018</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B35" s="92" t="s">
         <v>208</v>
       </c>
@@ -4209,7 +4222,7 @@
         <v>0.12500000000000003</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="12" thickBot="1">
+    <row r="36" spans="1:5" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B36" s="96" t="s">
         <v>211</v>
       </c>
@@ -4225,7 +4238,7 @@
         <v>1.4999999999999998</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B37" s="100" t="s">
         <v>212</v>
       </c>
@@ -4240,15 +4253,15 @@
         <v>7.4999999999999997E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C38" s="86"/>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B39" s="20" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B40" s="117" t="s">
         <v>215</v>
       </c>
@@ -4256,7 +4269,7 @@
       <c r="D40" s="117"/>
       <c r="E40" s="117"/>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B41" s="116" t="s">
         <v>231</v>
       </c>
@@ -4264,7 +4277,7 @@
       <c r="D41" s="117"/>
       <c r="E41" s="117"/>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B42" s="116" t="s">
         <v>229</v>
       </c>
@@ -4272,7 +4285,7 @@
       <c r="D42" s="117"/>
       <c r="E42" s="117"/>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B43" s="116" t="s">
         <v>230</v>
       </c>
@@ -4280,7 +4293,7 @@
       <c r="D43" s="116"/>
       <c r="E43" s="116"/>
     </row>
-    <row r="44" spans="1:5" ht="46.5" customHeight="1">
+    <row r="44" spans="1:5" ht="46.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B44" s="117" t="s">
         <v>157</v>
       </c>
@@ -4288,7 +4301,7 @@
       <c r="D44" s="117"/>
       <c r="E44" s="117"/>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A46" s="21" t="s">
         <v>138</v>
       </c>
@@ -4297,7 +4310,7 @@
       <c r="D46" s="21"/>
       <c r="E46" s="21"/>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B48" s="117" t="s">
         <v>217</v>
       </c>
@@ -4305,12 +4318,12 @@
       <c r="D48" s="117"/>
       <c r="E48" s="117"/>
     </row>
-    <row r="50" spans="2:5">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B50" s="23" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="52" spans="2:5">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B52" s="43" t="s">
         <v>78</v>
       </c>
@@ -4320,7 +4333,7 @@
       <c r="D52" s="47"/>
       <c r="E52" s="47"/>
     </row>
-    <row r="53" spans="2:5">
+    <row r="53" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B53" s="26" t="s">
         <v>199</v>
       </c>
@@ -4330,7 +4343,7 @@
       <c r="D53" s="48"/>
       <c r="E53" s="46"/>
     </row>
-    <row r="54" spans="2:5">
+    <row r="54" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B54" s="26" t="s">
         <v>198</v>
       </c>
@@ -4340,7 +4353,7 @@
       <c r="D54" s="48"/>
       <c r="E54" s="46"/>
     </row>
-    <row r="55" spans="2:5">
+    <row r="55" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B55" s="26" t="s">
         <v>197</v>
       </c>
@@ -4352,12 +4365,12 @@
       </c>
       <c r="E55" s="46"/>
     </row>
-    <row r="57" spans="2:5">
+    <row r="57" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B57" s="23" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="59" spans="2:5">
+    <row r="59" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B59" s="43" t="s">
         <v>79</v>
       </c>
@@ -4371,7 +4384,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="60" spans="2:5">
+    <row r="60" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B60" s="26" t="s">
         <v>63</v>
       </c>
@@ -4385,7 +4398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="2:5">
+    <row r="61" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B61" s="26" t="s">
         <v>64</v>
       </c>
@@ -4399,7 +4412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="2:5">
+    <row r="62" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B62" s="26" t="s">
         <v>194</v>
       </c>
@@ -4413,7 +4426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="2:5">
+    <row r="63" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B63" s="26" t="s">
         <v>192</v>
       </c>
@@ -4427,7 +4440,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="2:5">
+    <row r="64" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B64" s="26" t="s">
         <v>193</v>
       </c>
@@ -4441,7 +4454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.15">
       <c r="D65" s="27" t="s">
         <v>71</v>
       </c>
@@ -4450,7 +4463,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="12" thickBot="1">
+    <row r="66" spans="1:5" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="D66" s="41" t="s">
         <v>140</v>
       </c>
@@ -4459,23 +4472,23 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="12" thickTop="1"/>
-    <row r="68" spans="1:5">
+    <row r="67" spans="1:5" ht="13" thickTop="1" x14ac:dyDescent="0.15"/>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B68" s="1" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B69" s="1" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B70" s="1" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A72" s="21" t="s">
         <v>72</v>
       </c>
@@ -4484,7 +4497,7 @@
       <c r="D72" s="21"/>
       <c r="E72" s="21"/>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B74" s="117" t="s">
         <v>139</v>
       </c>
@@ -4492,7 +4505,7 @@
       <c r="D74" s="117"/>
       <c r="E74" s="117"/>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A76" s="28" t="s">
         <v>60</v>
       </c>
@@ -4500,12 +4513,12 @@
         <v>221</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B77" s="24" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A79" s="28" t="s">
         <v>200</v>
       </c>
@@ -4513,13 +4526,13 @@
         <v>220</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B80" s="1" t="str">
         <f>B19</f>
         <v>- Only investments with ERB &gt; 0 and Market Price &lt;= Entry Price are eligible for portfolio allocation.</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B81" s="104" t="s">
         <v>224</v>
       </c>
@@ -4527,7 +4540,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B82" s="104" t="s">
         <v>223</v>
       </c>
@@ -4535,33 +4548,33 @@
         <v>191</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B83" s="103" t="str">
         <f>B20</f>
         <v>- Non-selected investments receive 50% of normal allocation.</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B85" s="20" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="86" spans="1:5">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B86" s="1" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B87" s="1" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="88" spans="1:5">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B88" s="1" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A90" s="21" t="s">
         <v>73</v>
       </c>
@@ -4570,22 +4583,22 @@
       <c r="D90" s="21"/>
       <c r="E90" s="21"/>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B92" s="20" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B93" s="24" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B94" s="24" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B95" s="24" t="s">
         <v>148</v>
       </c>
@@ -4615,9 +4628,9 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AA358"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="11.65"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="2.46484375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.5" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="18.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="8.6640625" style="2" customWidth="1"/>
@@ -4632,12 +4645,12 @@
     <col min="23" max="23" width="8.6640625" style="74" customWidth="1"/>
     <col min="24" max="24" width="8.6640625" style="1" customWidth="1"/>
     <col min="25" max="25" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.796875" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.796875" style="11"/>
-    <col min="28" max="16384" width="8.796875" style="1"/>
+    <col min="26" max="26" width="11.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.83203125" style="11"/>
+    <col min="28" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.15">
       <c r="A1" s="5"/>
       <c r="B1" s="6" t="s">
         <v>3</v>
@@ -4684,7 +4697,7 @@
       <c r="Z1" s="119"/>
       <c r="AA1" s="119"/>
     </row>
-    <row r="2" spans="1:27" ht="26" customHeight="1">
+    <row r="2" spans="1:27" ht="26" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B2" s="7" t="s">
         <v>2</v>
       </c>
@@ -4764,7 +4777,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:27">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B3" s="11" t="s">
         <v>333</v>
       </c>
@@ -4772,21 +4785,21 @@
         <v>334</v>
       </c>
       <c r="D3" s="2">
-        <v>55.39</v>
+        <v>55.74</v>
       </c>
       <c r="E3" s="12" t="s">
         <v>327</v>
       </c>
       <c r="F3" s="15">
-        <v>0.10145588872206046</v>
+        <v>9.9063779841966904E-2</v>
       </c>
       <c r="G3" s="15">
         <f>F3 - Portfolio_Mgmt!$C$10</f>
-        <v>1.4455888722060467E-2</v>
+        <v>1.206377984196691E-2</v>
       </c>
       <c r="H3" s="15">
         <f>F3 - Portfolio_Mgmt!$C$11</f>
-        <v>8.2455888722060458E-2</v>
+        <v>8.0063779841966901E-2</v>
       </c>
       <c r="I3" s="15">
         <v>0</v>
@@ -4807,10 +4820,10 @@
         <v>57.551879180502802</v>
       </c>
       <c r="O3" s="4">
-        <v>7.8335820589004693E-2</v>
+        <v>7.7843937969590424E-2</v>
       </c>
       <c r="P3" s="4">
-        <v>3.899620870193176E-2</v>
+        <v>3.8751345532831001E-2</v>
       </c>
       <c r="Q3" s="4">
         <v>1.2182305488640417</v>
@@ -4846,7 +4859,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="4" spans="1:27">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B4" s="11" t="s">
         <v>329</v>
       </c>
@@ -4854,21 +4867,21 @@
         <v>331</v>
       </c>
       <c r="D4" s="2">
-        <v>16.100000000000001</v>
+        <v>15.99</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>327</v>
       </c>
       <c r="F4" s="15">
-        <v>8.9439282299528022E-2</v>
+        <v>9.2071429726595877E-2</v>
       </c>
       <c r="G4" s="15">
         <f>F4 - Portfolio_Mgmt!$C$10</f>
-        <v>2.4392822995280283E-3</v>
+        <v>5.071429726595883E-3</v>
       </c>
       <c r="H4" s="15">
         <f>F4 - Portfolio_Mgmt!$C$11</f>
-        <v>7.0439282299528019E-2</v>
+        <v>7.3071429726595874E-2</v>
       </c>
       <c r="I4" s="15">
         <v>0</v>
@@ -4889,10 +4902,10 @@
         <v>16.202875796143875</v>
       </c>
       <c r="O4" s="4">
-        <v>7.3107035109274451E-2</v>
+        <v>7.3609960303897354E-2</v>
       </c>
       <c r="P4" s="4">
-        <v>5.9254658385093167E-2</v>
+        <v>5.966228893058162E-2</v>
       </c>
       <c r="Q4" s="4">
         <v>0.2026552385945618</v>
@@ -4928,7 +4941,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="5" spans="1:27">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B5" s="11" t="s">
         <v>341</v>
       </c>
@@ -4936,21 +4949,21 @@
         <v>342</v>
       </c>
       <c r="D5" s="2">
-        <v>10.28</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>327</v>
       </c>
       <c r="F5" s="15">
-        <v>7.8003271289299514E-2</v>
+        <v>8.0906602549356998E-2</v>
       </c>
       <c r="G5" s="15">
         <f>F5 - Portfolio_Mgmt!$C$10</f>
-        <v>-8.9967287107004801E-3</v>
+        <v>-6.0933974506429955E-3</v>
       </c>
       <c r="H5" s="15">
         <f>F5 - Portfolio_Mgmt!$C$11</f>
-        <v>5.9003271289299511E-2</v>
+        <v>6.1906602549356995E-2</v>
       </c>
       <c r="I5" s="15">
         <v>0</v>
@@ -4971,10 +4984,10 @@
         <v>10.034835914511921</v>
       </c>
       <c r="O5" s="4">
-        <v>3.4320466769170409E-2</v>
+        <v>3.4589646900693313E-2</v>
       </c>
       <c r="P5" s="4">
-        <v>3.5019455252918295E-2</v>
+        <v>3.529411764705883E-2</v>
       </c>
       <c r="Q5" s="4">
         <v>3.888300021475994E-2</v>
@@ -5010,7 +5023,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="6" spans="1:27">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B6" s="11" t="s">
         <v>344</v>
       </c>
@@ -5018,21 +5031,21 @@
         <v>345</v>
       </c>
       <c r="D6" s="2">
-        <v>5.73</v>
+        <v>5.71</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>327</v>
       </c>
       <c r="F6" s="15">
-        <v>5.3112503494364027E-2</v>
+        <v>5.4377980810659921E-2</v>
       </c>
       <c r="G6" s="15">
         <f>F6 - Portfolio_Mgmt!$C$10</f>
-        <v>-3.3887496505635967E-2</v>
+        <v>-3.2622019189340073E-2</v>
       </c>
       <c r="H6" s="15">
         <f>F6 - Portfolio_Mgmt!$C$11</f>
-        <v>3.4112503494364024E-2</v>
+        <v>3.5377980810659918E-2</v>
       </c>
       <c r="I6" s="15">
         <v>0</v>
@@ -5053,10 +5066,10 @@
         <v>5.225618425612172</v>
       </c>
       <c r="O6" s="4">
-        <v>4.0139632953133386E-2</v>
+        <v>4.0280227114090073E-2</v>
       </c>
       <c r="P6" s="4">
-        <v>3.1570680628272244E-2</v>
+        <v>3.1681260945709278E-2</v>
       </c>
       <c r="Q6" s="4">
         <v>4.9029562887232557E-2</v>
@@ -5092,7 +5105,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="7" spans="1:27">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B7" s="11" t="s">
         <v>337</v>
       </c>
@@ -5100,21 +5113,21 @@
         <v>338</v>
       </c>
       <c r="D7" s="2">
-        <v>22.74</v>
+        <v>22.78</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>327</v>
       </c>
       <c r="F7" s="15">
-        <v>4.6547136992241445E-2</v>
+        <v>4.590904453268374E-2</v>
       </c>
       <c r="G7" s="15">
         <f>F7 - Portfolio_Mgmt!$C$10</f>
-        <v>-4.0452863007758549E-2</v>
+        <v>-4.1090955467316254E-2</v>
       </c>
       <c r="H7" s="15">
         <f>F7 - Portfolio_Mgmt!$C$11</f>
-        <v>2.7547136992241445E-2</v>
+        <v>2.6909044532683741E-2</v>
       </c>
       <c r="I7" s="15">
         <v>0</v>
@@ -5135,10 +5148,10 @@
         <v>20.388648577016472</v>
       </c>
       <c r="O7" s="4">
-        <v>5.8234869031407205E-2</v>
+        <v>5.8132612896145734E-2</v>
       </c>
       <c r="P7" s="4">
-        <v>4.1952506596306074E-2</v>
+        <v>4.1878841088674276E-2</v>
       </c>
       <c r="Q7" s="4">
         <v>0.15648173464349882</v>
@@ -5174,7 +5187,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="8" spans="1:27">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B8" s="11" t="s">
         <v>339</v>
       </c>
@@ -5182,21 +5195,21 @@
         <v>340</v>
       </c>
       <c r="D8" s="2">
-        <v>68.88</v>
+        <v>70.25</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>327</v>
       </c>
       <c r="F8" s="15">
-        <v>4.4158785780313403E-2</v>
+        <v>3.6914739540422126E-2</v>
       </c>
       <c r="G8" s="15">
         <f>F8 - Portfolio_Mgmt!$C$10</f>
-        <v>-4.2841214219686591E-2</v>
+        <v>-5.0085260459577868E-2</v>
       </c>
       <c r="H8" s="15">
         <f>F8 - Portfolio_Mgmt!$C$11</f>
-        <v>2.5158785780313404E-2</v>
+        <v>1.7914739540422126E-2</v>
       </c>
       <c r="I8" s="15">
         <v>0</v>
@@ -5217,10 +5230,10 @@
         <v>61.489408566601746</v>
       </c>
       <c r="O8" s="4">
-        <v>5.2546092846258032E-2</v>
+        <v>5.1521350537370156E-2</v>
       </c>
       <c r="P8" s="4">
-        <v>6.071864111498259E-2</v>
+        <v>5.9534519572953748E-2</v>
       </c>
       <c r="Q8" s="4">
         <v>0.14093304007128551</v>
@@ -5256,7 +5269,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="9" spans="1:27">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B9" s="11" t="s">
         <v>347</v>
       </c>
@@ -5264,21 +5277,21 @@
         <v>348</v>
       </c>
       <c r="D9" s="2">
-        <v>20.53</v>
+        <v>20.55</v>
       </c>
       <c r="E9" s="12" t="s">
         <v>327</v>
       </c>
       <c r="F9" s="15">
-        <v>2.002653273777133E-2</v>
+        <v>1.9679211078303283E-2</v>
       </c>
       <c r="G9" s="15">
         <f>F9 - Portfolio_Mgmt!$C$10</f>
-        <v>-6.6973467262228664E-2</v>
+        <v>-6.7320788921696711E-2</v>
       </c>
       <c r="H9" s="15">
         <f>F9 - Portfolio_Mgmt!$C$11</f>
-        <v>1.0265327377713303E-3</v>
+        <v>6.7921107830328301E-4</v>
       </c>
       <c r="I9" s="15">
         <v>0</v>
@@ -5299,10 +5312,10 @@
         <v>17.124648599063175</v>
       </c>
       <c r="O9" s="4">
-        <v>5.2715283675273471E-2</v>
+        <v>5.2663979262937442E-2</v>
       </c>
       <c r="P9" s="4">
-        <v>4.8222113979542139E-2</v>
+        <v>4.817518248175183E-2</v>
       </c>
       <c r="Q9" s="4">
         <v>0.15161114820375229</v>
@@ -5338,7 +5351,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="10" spans="1:27">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B10" s="11" t="s">
         <v>328</v>
       </c>
@@ -5346,21 +5359,21 @@
         <v>349</v>
       </c>
       <c r="D10" s="2">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>327</v>
       </c>
       <c r="F10" s="15">
-        <v>1.5510765594796805E-2</v>
+        <v>1.7070987343137611E-2</v>
       </c>
       <c r="G10" s="15">
         <f>F10 - Portfolio_Mgmt!$C$10</f>
-        <v>-7.1489234405203189E-2</v>
+        <v>-6.9929012656862383E-2</v>
       </c>
       <c r="H10" s="15">
         <f>F10 - Portfolio_Mgmt!$C$11</f>
-        <v>-3.4892344052031947E-3</v>
+        <v>-1.9290126568623882E-3</v>
       </c>
       <c r="I10" s="15">
         <v>0</v>
@@ -5381,10 +5394,10 @@
         <v>18.773924722806626</v>
       </c>
       <c r="O10" s="4">
-        <v>0.24216518916613325</v>
+        <v>0.24323199616686514</v>
       </c>
       <c r="P10" s="4">
-        <v>4.6491228070175437E-2</v>
+        <v>4.6696035242290754E-2</v>
       </c>
       <c r="Q10" s="4">
         <v>0.17249144202566888</v>
@@ -5420,7 +5433,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="11" spans="1:27">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B11" s="11" t="s">
         <v>335</v>
       </c>
@@ -5428,21 +5441,21 @@
         <v>336</v>
       </c>
       <c r="D11" s="2">
-        <v>53.23</v>
+        <v>53.31</v>
       </c>
       <c r="E11" s="12" t="s">
         <v>327</v>
       </c>
       <c r="F11" s="15">
-        <v>1.3156769539393265E-2</v>
+        <v>1.2641153933681482E-2</v>
       </c>
       <c r="G11" s="15">
         <f>F11 - Portfolio_Mgmt!$C$10</f>
-        <v>-7.3843230460606729E-2</v>
+        <v>-7.4358846066318512E-2</v>
       </c>
       <c r="H11" s="15">
         <f>F11 - Portfolio_Mgmt!$C$11</f>
-        <v>-5.8432304606067346E-3</v>
+        <v>-6.358846066318518E-3</v>
       </c>
       <c r="I11" s="15">
         <v>0</v>
@@ -5463,10 +5476,10 @@
         <v>43.262452230628902</v>
       </c>
       <c r="O11" s="4">
-        <v>4.0634591593908677E-2</v>
+        <v>4.0573613028395392E-2</v>
       </c>
       <c r="P11" s="4">
-        <v>1.690775878264137E-2</v>
+        <v>1.6882386043894203E-2</v>
       </c>
       <c r="Q11" s="4">
         <v>0.14549955248916155</v>
@@ -5502,7 +5515,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="12" spans="1:27">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B12" s="11" t="s">
         <v>351</v>
       </c>
@@ -5510,21 +5523,21 @@
         <v>352</v>
       </c>
       <c r="D12" s="2">
-        <v>15.57</v>
+        <v>15.45</v>
       </c>
       <c r="E12" s="12" t="s">
         <v>327</v>
       </c>
       <c r="F12" s="15">
-        <v>-0.14806866552364339</v>
+        <v>-0.14580344670318324</v>
       </c>
       <c r="G12" s="15">
         <f>F12 - Portfolio_Mgmt!$C$10</f>
-        <v>-0.23506866552364339</v>
+        <v>-0.23280344670318323</v>
       </c>
       <c r="H12" s="15">
         <f>F12 - Portfolio_Mgmt!$C$11</f>
-        <v>-0.16706866552364338</v>
+        <v>-0.16480344670318323</v>
       </c>
       <c r="I12" s="15">
         <v>0</v>
@@ -5545,10 +5558,10 @@
         <v>7.6893682545464594</v>
       </c>
       <c r="O12" s="4">
-        <v>2.8493267176075268E-2</v>
+        <v>2.8714574105598186E-2</v>
       </c>
       <c r="P12" s="4">
-        <v>2.3121387283236997E-2</v>
+        <v>2.3300970873786412E-2</v>
       </c>
       <c r="Q12" s="4">
         <v>7.1587241945726146E-2</v>
@@ -5584,7 +5597,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="13" spans="1:27">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
       <c r="E13" s="12"/>
@@ -5597,7 +5610,7 @@
       <c r="Z13" s="14"/>
       <c r="AA13" s="16"/>
     </row>
-    <row r="14" spans="1:27">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
       <c r="E14" s="12"/>
@@ -5610,7 +5623,7 @@
       <c r="Z14" s="14"/>
       <c r="AA14" s="16"/>
     </row>
-    <row r="15" spans="1:27">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
       <c r="E15" s="12"/>
@@ -5623,7 +5636,7 @@
       <c r="Z15" s="14"/>
       <c r="AA15" s="16"/>
     </row>
-    <row r="16" spans="1:27">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.15">
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
       <c r="E16" s="12"/>
@@ -5636,7 +5649,7 @@
       <c r="Z16" s="14"/>
       <c r="AA16" s="16"/>
     </row>
-    <row r="17" spans="2:26">
+    <row r="17" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
       <c r="E17" s="12"/>
@@ -5648,7 +5661,7 @@
       <c r="Y17" s="11"/>
       <c r="Z17" s="14"/>
     </row>
-    <row r="18" spans="2:26">
+    <row r="18" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
       <c r="E18" s="12"/>
@@ -5660,7 +5673,7 @@
       <c r="Y18" s="11"/>
       <c r="Z18" s="14"/>
     </row>
-    <row r="19" spans="2:26">
+    <row r="19" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
       <c r="E19" s="12"/>
@@ -5672,7 +5685,7 @@
       <c r="Y19" s="11"/>
       <c r="Z19" s="14"/>
     </row>
-    <row r="20" spans="2:26">
+    <row r="20" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
       <c r="E20" s="12"/>
@@ -5684,7 +5697,7 @@
       <c r="Y20" s="11"/>
       <c r="Z20" s="14"/>
     </row>
-    <row r="21" spans="2:26">
+    <row r="21" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
       <c r="E21" s="12"/>
@@ -5696,7 +5709,7 @@
       <c r="Y21" s="11"/>
       <c r="Z21" s="14"/>
     </row>
-    <row r="22" spans="2:26">
+    <row r="22" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
       <c r="E22" s="12"/>
@@ -5708,7 +5721,7 @@
       <c r="Y22" s="11"/>
       <c r="Z22" s="14"/>
     </row>
-    <row r="23" spans="2:26">
+    <row r="23" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
       <c r="E23" s="12"/>
@@ -5720,7 +5733,7 @@
       <c r="Y23" s="11"/>
       <c r="Z23" s="14"/>
     </row>
-    <row r="24" spans="2:26">
+    <row r="24" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
       <c r="E24" s="12"/>
@@ -5732,7 +5745,7 @@
       <c r="Y24" s="11"/>
       <c r="Z24" s="14"/>
     </row>
-    <row r="25" spans="2:26">
+    <row r="25" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
       <c r="E25" s="12"/>
@@ -5744,7 +5757,7 @@
       <c r="Y25" s="11"/>
       <c r="Z25" s="14"/>
     </row>
-    <row r="26" spans="2:26">
+    <row r="26" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
       <c r="E26" s="12"/>
@@ -5756,7 +5769,7 @@
       <c r="Y26" s="11"/>
       <c r="Z26" s="14"/>
     </row>
-    <row r="27" spans="2:26">
+    <row r="27" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
       <c r="E27" s="12"/>
@@ -5768,7 +5781,7 @@
       <c r="Y27" s="11"/>
       <c r="Z27" s="14"/>
     </row>
-    <row r="28" spans="2:26">
+    <row r="28" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
       <c r="E28" s="12"/>
@@ -5780,7 +5793,7 @@
       <c r="Y28" s="11"/>
       <c r="Z28" s="14"/>
     </row>
-    <row r="29" spans="2:26">
+    <row r="29" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
       <c r="E29" s="12"/>
@@ -5792,7 +5805,7 @@
       <c r="Y29" s="11"/>
       <c r="Z29" s="14"/>
     </row>
-    <row r="30" spans="2:26">
+    <row r="30" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
       <c r="E30" s="12"/>
@@ -5804,7 +5817,7 @@
       <c r="Y30" s="11"/>
       <c r="Z30" s="14"/>
     </row>
-    <row r="31" spans="2:26">
+    <row r="31" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
       <c r="E31" s="12"/>
@@ -5816,7 +5829,7 @@
       <c r="Y31" s="11"/>
       <c r="Z31" s="14"/>
     </row>
-    <row r="32" spans="2:26">
+    <row r="32" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
       <c r="E32" s="12"/>
@@ -5828,7 +5841,7 @@
       <c r="Y32" s="11"/>
       <c r="Z32" s="14"/>
     </row>
-    <row r="33" spans="2:26">
+    <row r="33" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
       <c r="E33" s="12"/>
@@ -5840,7 +5853,7 @@
       <c r="Y33" s="11"/>
       <c r="Z33" s="14"/>
     </row>
-    <row r="34" spans="2:26">
+    <row r="34" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
       <c r="E34" s="12"/>
@@ -5852,7 +5865,7 @@
       <c r="Y34" s="11"/>
       <c r="Z34" s="14"/>
     </row>
-    <row r="35" spans="2:26">
+    <row r="35" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B35" s="11"/>
       <c r="C35" s="11"/>
       <c r="E35" s="12"/>
@@ -5864,7 +5877,7 @@
       <c r="Y35" s="11"/>
       <c r="Z35" s="14"/>
     </row>
-    <row r="36" spans="2:26">
+    <row r="36" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
       <c r="E36" s="12"/>
@@ -5876,7 +5889,7 @@
       <c r="Y36" s="11"/>
       <c r="Z36" s="14"/>
     </row>
-    <row r="37" spans="2:26">
+    <row r="37" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B37" s="11"/>
       <c r="C37" s="11"/>
       <c r="E37" s="12"/>
@@ -5888,7 +5901,7 @@
       <c r="Y37" s="11"/>
       <c r="Z37" s="14"/>
     </row>
-    <row r="38" spans="2:26">
+    <row r="38" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B38" s="11"/>
       <c r="C38" s="11"/>
       <c r="E38" s="12"/>
@@ -5900,7 +5913,7 @@
       <c r="Y38" s="11"/>
       <c r="Z38" s="14"/>
     </row>
-    <row r="39" spans="2:26">
+    <row r="39" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B39" s="11"/>
       <c r="C39" s="11"/>
       <c r="E39" s="12"/>
@@ -5912,7 +5925,7 @@
       <c r="Y39" s="11"/>
       <c r="Z39" s="14"/>
     </row>
-    <row r="40" spans="2:26">
+    <row r="40" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B40" s="11"/>
       <c r="C40" s="11"/>
       <c r="E40" s="12"/>
@@ -5924,7 +5937,7 @@
       <c r="Y40" s="11"/>
       <c r="Z40" s="14"/>
     </row>
-    <row r="41" spans="2:26">
+    <row r="41" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B41" s="11"/>
       <c r="C41" s="11"/>
       <c r="E41" s="12"/>
@@ -5936,7 +5949,7 @@
       <c r="Y41" s="11"/>
       <c r="Z41" s="14"/>
     </row>
-    <row r="42" spans="2:26">
+    <row r="42" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B42" s="11"/>
       <c r="C42" s="11"/>
       <c r="E42" s="12"/>
@@ -5948,7 +5961,7 @@
       <c r="Y42" s="11"/>
       <c r="Z42" s="14"/>
     </row>
-    <row r="43" spans="2:26">
+    <row r="43" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B43" s="11"/>
       <c r="C43" s="11"/>
       <c r="E43" s="12"/>
@@ -5960,7 +5973,7 @@
       <c r="Y43" s="11"/>
       <c r="Z43" s="14"/>
     </row>
-    <row r="44" spans="2:26">
+    <row r="44" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B44" s="11"/>
       <c r="C44" s="11"/>
       <c r="E44" s="12"/>
@@ -5972,7 +5985,7 @@
       <c r="Y44" s="11"/>
       <c r="Z44" s="14"/>
     </row>
-    <row r="45" spans="2:26">
+    <row r="45" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B45" s="11"/>
       <c r="C45" s="11"/>
       <c r="E45" s="12"/>
@@ -5984,7 +5997,7 @@
       <c r="Y45" s="11"/>
       <c r="Z45" s="14"/>
     </row>
-    <row r="46" spans="2:26">
+    <row r="46" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B46" s="11"/>
       <c r="C46" s="11"/>
       <c r="E46" s="12"/>
@@ -5996,7 +6009,7 @@
       <c r="Y46" s="11"/>
       <c r="Z46" s="14"/>
     </row>
-    <row r="47" spans="2:26">
+    <row r="47" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B47" s="11"/>
       <c r="C47" s="11"/>
       <c r="E47" s="12"/>
@@ -6008,7 +6021,7 @@
       <c r="Y47" s="11"/>
       <c r="Z47" s="14"/>
     </row>
-    <row r="48" spans="2:26">
+    <row r="48" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
       <c r="E48" s="12"/>
@@ -6020,7 +6033,7 @@
       <c r="Y48" s="11"/>
       <c r="Z48" s="14"/>
     </row>
-    <row r="49" spans="2:26">
+    <row r="49" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B49" s="11"/>
       <c r="C49" s="11"/>
       <c r="E49" s="12"/>
@@ -6032,7 +6045,7 @@
       <c r="Y49" s="11"/>
       <c r="Z49" s="14"/>
     </row>
-    <row r="50" spans="2:26">
+    <row r="50" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B50" s="11"/>
       <c r="C50" s="11"/>
       <c r="E50" s="12"/>
@@ -6044,7 +6057,7 @@
       <c r="Y50" s="11"/>
       <c r="Z50" s="14"/>
     </row>
-    <row r="51" spans="2:26">
+    <row r="51" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B51" s="11"/>
       <c r="C51" s="11"/>
       <c r="E51" s="12"/>
@@ -6056,7 +6069,7 @@
       <c r="Y51" s="11"/>
       <c r="Z51" s="14"/>
     </row>
-    <row r="52" spans="2:26">
+    <row r="52" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B52" s="11"/>
       <c r="C52" s="11"/>
       <c r="E52" s="12"/>
@@ -6068,7 +6081,7 @@
       <c r="Y52" s="11"/>
       <c r="Z52" s="14"/>
     </row>
-    <row r="53" spans="2:26">
+    <row r="53" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B53" s="11"/>
       <c r="C53" s="11"/>
       <c r="E53" s="12"/>
@@ -6080,7 +6093,7 @@
       <c r="Y53" s="11"/>
       <c r="Z53" s="14"/>
     </row>
-    <row r="54" spans="2:26">
+    <row r="54" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B54" s="11"/>
       <c r="C54" s="11"/>
       <c r="E54" s="12"/>
@@ -6092,7 +6105,7 @@
       <c r="Y54" s="11"/>
       <c r="Z54" s="14"/>
     </row>
-    <row r="55" spans="2:26">
+    <row r="55" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B55" s="11"/>
       <c r="C55" s="11"/>
       <c r="E55" s="12"/>
@@ -6104,7 +6117,7 @@
       <c r="Y55" s="11"/>
       <c r="Z55" s="14"/>
     </row>
-    <row r="56" spans="2:26">
+    <row r="56" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B56" s="11"/>
       <c r="C56" s="11"/>
       <c r="E56" s="12"/>
@@ -6116,7 +6129,7 @@
       <c r="Y56" s="11"/>
       <c r="Z56" s="14"/>
     </row>
-    <row r="57" spans="2:26">
+    <row r="57" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B57" s="11"/>
       <c r="C57" s="11"/>
       <c r="E57" s="12"/>
@@ -6128,7 +6141,7 @@
       <c r="Y57" s="11"/>
       <c r="Z57" s="14"/>
     </row>
-    <row r="58" spans="2:26">
+    <row r="58" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B58" s="11"/>
       <c r="C58" s="11"/>
       <c r="E58" s="12"/>
@@ -6140,7 +6153,7 @@
       <c r="Y58" s="11"/>
       <c r="Z58" s="14"/>
     </row>
-    <row r="59" spans="2:26">
+    <row r="59" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B59" s="11"/>
       <c r="C59" s="11"/>
       <c r="E59" s="12"/>
@@ -6152,7 +6165,7 @@
       <c r="Y59" s="11"/>
       <c r="Z59" s="14"/>
     </row>
-    <row r="60" spans="2:26">
+    <row r="60" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B60" s="11"/>
       <c r="C60" s="11"/>
       <c r="E60" s="12"/>
@@ -6164,7 +6177,7 @@
       <c r="Y60" s="11"/>
       <c r="Z60" s="14"/>
     </row>
-    <row r="61" spans="2:26">
+    <row r="61" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B61" s="11"/>
       <c r="C61" s="11"/>
       <c r="E61" s="12"/>
@@ -6176,7 +6189,7 @@
       <c r="Y61" s="11"/>
       <c r="Z61" s="14"/>
     </row>
-    <row r="62" spans="2:26">
+    <row r="62" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B62" s="11"/>
       <c r="C62" s="11"/>
       <c r="E62" s="12"/>
@@ -6188,7 +6201,7 @@
       <c r="Y62" s="11"/>
       <c r="Z62" s="14"/>
     </row>
-    <row r="63" spans="2:26">
+    <row r="63" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B63" s="11"/>
       <c r="C63" s="11"/>
       <c r="E63" s="12"/>
@@ -6200,7 +6213,7 @@
       <c r="Y63" s="11"/>
       <c r="Z63" s="14"/>
     </row>
-    <row r="64" spans="2:26">
+    <row r="64" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B64" s="11"/>
       <c r="C64" s="11"/>
       <c r="E64" s="12"/>
@@ -6212,7 +6225,7 @@
       <c r="Y64" s="11"/>
       <c r="Z64" s="14"/>
     </row>
-    <row r="65" spans="2:26">
+    <row r="65" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B65" s="11"/>
       <c r="C65" s="11"/>
       <c r="E65" s="12"/>
@@ -6224,7 +6237,7 @@
       <c r="Y65" s="11"/>
       <c r="Z65" s="14"/>
     </row>
-    <row r="66" spans="2:26">
+    <row r="66" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B66" s="11"/>
       <c r="C66" s="11"/>
       <c r="E66" s="12"/>
@@ -6236,7 +6249,7 @@
       <c r="Y66" s="11"/>
       <c r="Z66" s="14"/>
     </row>
-    <row r="67" spans="2:26">
+    <row r="67" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B67" s="11"/>
       <c r="C67" s="11"/>
       <c r="E67" s="12"/>
@@ -6248,7 +6261,7 @@
       <c r="Y67" s="11"/>
       <c r="Z67" s="14"/>
     </row>
-    <row r="68" spans="2:26">
+    <row r="68" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B68" s="11"/>
       <c r="C68" s="11"/>
       <c r="E68" s="12"/>
@@ -6260,7 +6273,7 @@
       <c r="Y68" s="11"/>
       <c r="Z68" s="14"/>
     </row>
-    <row r="69" spans="2:26">
+    <row r="69" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B69" s="11"/>
       <c r="C69" s="11"/>
       <c r="E69" s="12"/>
@@ -6272,7 +6285,7 @@
       <c r="Y69" s="11"/>
       <c r="Z69" s="14"/>
     </row>
-    <row r="70" spans="2:26">
+    <row r="70" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B70" s="11"/>
       <c r="C70" s="11"/>
       <c r="E70" s="12"/>
@@ -6284,7 +6297,7 @@
       <c r="Y70" s="11"/>
       <c r="Z70" s="14"/>
     </row>
-    <row r="71" spans="2:26">
+    <row r="71" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B71" s="11"/>
       <c r="C71" s="11"/>
       <c r="E71" s="12"/>
@@ -6296,7 +6309,7 @@
       <c r="Y71" s="11"/>
       <c r="Z71" s="14"/>
     </row>
-    <row r="72" spans="2:26">
+    <row r="72" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B72" s="11"/>
       <c r="C72" s="11"/>
       <c r="E72" s="12"/>
@@ -6308,7 +6321,7 @@
       <c r="Y72" s="11"/>
       <c r="Z72" s="14"/>
     </row>
-    <row r="73" spans="2:26">
+    <row r="73" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B73" s="11"/>
       <c r="C73" s="11"/>
       <c r="E73" s="12"/>
@@ -6320,7 +6333,7 @@
       <c r="Y73" s="11"/>
       <c r="Z73" s="14"/>
     </row>
-    <row r="74" spans="2:26">
+    <row r="74" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B74" s="11"/>
       <c r="C74" s="11"/>
       <c r="E74" s="12"/>
@@ -6332,7 +6345,7 @@
       <c r="Y74" s="11"/>
       <c r="Z74" s="14"/>
     </row>
-    <row r="75" spans="2:26">
+    <row r="75" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B75" s="11"/>
       <c r="C75" s="11"/>
       <c r="E75" s="12"/>
@@ -6344,7 +6357,7 @@
       <c r="Y75" s="11"/>
       <c r="Z75" s="14"/>
     </row>
-    <row r="76" spans="2:26">
+    <row r="76" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B76" s="11"/>
       <c r="C76" s="11"/>
       <c r="E76" s="12"/>
@@ -6356,7 +6369,7 @@
       <c r="Y76" s="11"/>
       <c r="Z76" s="14"/>
     </row>
-    <row r="77" spans="2:26">
+    <row r="77" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B77" s="11"/>
       <c r="C77" s="11"/>
       <c r="E77" s="12"/>
@@ -6368,7 +6381,7 @@
       <c r="Y77" s="11"/>
       <c r="Z77" s="14"/>
     </row>
-    <row r="78" spans="2:26">
+    <row r="78" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B78" s="11"/>
       <c r="C78" s="11"/>
       <c r="E78" s="12"/>
@@ -6380,7 +6393,7 @@
       <c r="Y78" s="11"/>
       <c r="Z78" s="14"/>
     </row>
-    <row r="79" spans="2:26">
+    <row r="79" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B79" s="11"/>
       <c r="C79" s="11"/>
       <c r="E79" s="12"/>
@@ -6392,7 +6405,7 @@
       <c r="Y79" s="11"/>
       <c r="Z79" s="14"/>
     </row>
-    <row r="80" spans="2:26">
+    <row r="80" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B80" s="11"/>
       <c r="C80" s="11"/>
       <c r="E80" s="12"/>
@@ -6404,7 +6417,7 @@
       <c r="Y80" s="11"/>
       <c r="Z80" s="14"/>
     </row>
-    <row r="81" spans="2:26">
+    <row r="81" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B81" s="11"/>
       <c r="C81" s="11"/>
       <c r="E81" s="12"/>
@@ -6416,7 +6429,7 @@
       <c r="Y81" s="11"/>
       <c r="Z81" s="14"/>
     </row>
-    <row r="82" spans="2:26">
+    <row r="82" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B82" s="11"/>
       <c r="C82" s="11"/>
       <c r="E82" s="12"/>
@@ -6428,7 +6441,7 @@
       <c r="Y82" s="11"/>
       <c r="Z82" s="14"/>
     </row>
-    <row r="83" spans="2:26">
+    <row r="83" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B83" s="11"/>
       <c r="C83" s="11"/>
       <c r="E83" s="12"/>
@@ -6440,7 +6453,7 @@
       <c r="Y83" s="11"/>
       <c r="Z83" s="14"/>
     </row>
-    <row r="84" spans="2:26">
+    <row r="84" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B84" s="11"/>
       <c r="C84" s="11"/>
       <c r="E84" s="12"/>
@@ -6452,7 +6465,7 @@
       <c r="Y84" s="11"/>
       <c r="Z84" s="14"/>
     </row>
-    <row r="85" spans="2:26">
+    <row r="85" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B85" s="11"/>
       <c r="C85" s="11"/>
       <c r="E85" s="12"/>
@@ -6464,7 +6477,7 @@
       <c r="Y85" s="11"/>
       <c r="Z85" s="14"/>
     </row>
-    <row r="86" spans="2:26">
+    <row r="86" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B86" s="11"/>
       <c r="C86" s="11"/>
       <c r="E86" s="12"/>
@@ -6476,7 +6489,7 @@
       <c r="Y86" s="11"/>
       <c r="Z86" s="14"/>
     </row>
-    <row r="87" spans="2:26">
+    <row r="87" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B87" s="11"/>
       <c r="C87" s="11"/>
       <c r="E87" s="12"/>
@@ -6488,7 +6501,7 @@
       <c r="Y87" s="11"/>
       <c r="Z87" s="14"/>
     </row>
-    <row r="88" spans="2:26">
+    <row r="88" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B88" s="11"/>
       <c r="C88" s="11"/>
       <c r="E88" s="12"/>
@@ -6500,7 +6513,7 @@
       <c r="Y88" s="11"/>
       <c r="Z88" s="14"/>
     </row>
-    <row r="89" spans="2:26">
+    <row r="89" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B89" s="11"/>
       <c r="C89" s="11"/>
       <c r="E89" s="12"/>
@@ -6512,7 +6525,7 @@
       <c r="Y89" s="11"/>
       <c r="Z89" s="14"/>
     </row>
-    <row r="90" spans="2:26">
+    <row r="90" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B90" s="11"/>
       <c r="C90" s="11"/>
       <c r="E90" s="12"/>
@@ -6524,7 +6537,7 @@
       <c r="Y90" s="11"/>
       <c r="Z90" s="14"/>
     </row>
-    <row r="91" spans="2:26">
+    <row r="91" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B91" s="11"/>
       <c r="C91" s="11"/>
       <c r="E91" s="12"/>
@@ -6536,7 +6549,7 @@
       <c r="Y91" s="11"/>
       <c r="Z91" s="14"/>
     </row>
-    <row r="92" spans="2:26">
+    <row r="92" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B92" s="11"/>
       <c r="C92" s="11"/>
       <c r="E92" s="12"/>
@@ -6548,7 +6561,7 @@
       <c r="Y92" s="11"/>
       <c r="Z92" s="14"/>
     </row>
-    <row r="93" spans="2:26">
+    <row r="93" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B93" s="11"/>
       <c r="C93" s="11"/>
       <c r="E93" s="12"/>
@@ -6560,7 +6573,7 @@
       <c r="Y93" s="11"/>
       <c r="Z93" s="14"/>
     </row>
-    <row r="94" spans="2:26">
+    <row r="94" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B94" s="11"/>
       <c r="C94" s="11"/>
       <c r="E94" s="12"/>
@@ -6572,7 +6585,7 @@
       <c r="Y94" s="11"/>
       <c r="Z94" s="14"/>
     </row>
-    <row r="95" spans="2:26">
+    <row r="95" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B95" s="11"/>
       <c r="C95" s="11"/>
       <c r="E95" s="12"/>
@@ -6584,7 +6597,7 @@
       <c r="Y95" s="11"/>
       <c r="Z95" s="14"/>
     </row>
-    <row r="96" spans="2:26">
+    <row r="96" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B96" s="11"/>
       <c r="C96" s="11"/>
       <c r="E96" s="12"/>
@@ -6596,7 +6609,7 @@
       <c r="Y96" s="11"/>
       <c r="Z96" s="14"/>
     </row>
-    <row r="97" spans="2:26">
+    <row r="97" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B97" s="11"/>
       <c r="C97" s="11"/>
       <c r="E97" s="12"/>
@@ -6608,7 +6621,7 @@
       <c r="Y97" s="11"/>
       <c r="Z97" s="14"/>
     </row>
-    <row r="98" spans="2:26">
+    <row r="98" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B98" s="11"/>
       <c r="C98" s="11"/>
       <c r="E98" s="12"/>
@@ -6620,7 +6633,7 @@
       <c r="Y98" s="11"/>
       <c r="Z98" s="14"/>
     </row>
-    <row r="99" spans="2:26">
+    <row r="99" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B99" s="11"/>
       <c r="C99" s="11"/>
       <c r="E99" s="12"/>
@@ -6632,7 +6645,7 @@
       <c r="Y99" s="11"/>
       <c r="Z99" s="14"/>
     </row>
-    <row r="100" spans="2:26">
+    <row r="100" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B100" s="11"/>
       <c r="C100" s="11"/>
       <c r="E100" s="12"/>
@@ -6644,7 +6657,7 @@
       <c r="Y100" s="11"/>
       <c r="Z100" s="14"/>
     </row>
-    <row r="101" spans="2:26">
+    <row r="101" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B101" s="11"/>
       <c r="C101" s="11"/>
       <c r="E101" s="12"/>
@@ -6656,7 +6669,7 @@
       <c r="Y101" s="11"/>
       <c r="Z101" s="14"/>
     </row>
-    <row r="102" spans="2:26">
+    <row r="102" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B102" s="11"/>
       <c r="C102" s="11"/>
       <c r="E102" s="12"/>
@@ -6668,7 +6681,7 @@
       <c r="Y102" s="11"/>
       <c r="Z102" s="14"/>
     </row>
-    <row r="103" spans="2:26">
+    <row r="103" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B103" s="11"/>
       <c r="C103" s="11"/>
       <c r="E103" s="12"/>
@@ -6680,7 +6693,7 @@
       <c r="Y103" s="11"/>
       <c r="Z103" s="14"/>
     </row>
-    <row r="104" spans="2:26">
+    <row r="104" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B104" s="11"/>
       <c r="C104" s="11"/>
       <c r="E104" s="12"/>
@@ -6692,7 +6705,7 @@
       <c r="Y104" s="11"/>
       <c r="Z104" s="14"/>
     </row>
-    <row r="105" spans="2:26">
+    <row r="105" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B105" s="11"/>
       <c r="C105" s="11"/>
       <c r="E105" s="12"/>
@@ -6704,7 +6717,7 @@
       <c r="Y105" s="11"/>
       <c r="Z105" s="14"/>
     </row>
-    <row r="106" spans="2:26">
+    <row r="106" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B106" s="11"/>
       <c r="C106" s="11"/>
       <c r="E106" s="12"/>
@@ -6716,7 +6729,7 @@
       <c r="Y106" s="11"/>
       <c r="Z106" s="14"/>
     </row>
-    <row r="107" spans="2:26">
+    <row r="107" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B107" s="11"/>
       <c r="C107" s="11"/>
       <c r="E107" s="12"/>
@@ -6728,7 +6741,7 @@
       <c r="Y107" s="11"/>
       <c r="Z107" s="14"/>
     </row>
-    <row r="108" spans="2:26">
+    <row r="108" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B108" s="11"/>
       <c r="C108" s="11"/>
       <c r="E108" s="12"/>
@@ -6740,7 +6753,7 @@
       <c r="Y108" s="11"/>
       <c r="Z108" s="14"/>
     </row>
-    <row r="109" spans="2:26">
+    <row r="109" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B109" s="11"/>
       <c r="C109" s="11"/>
       <c r="E109" s="12"/>
@@ -6752,7 +6765,7 @@
       <c r="Y109" s="11"/>
       <c r="Z109" s="14"/>
     </row>
-    <row r="110" spans="2:26">
+    <row r="110" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B110" s="11"/>
       <c r="C110" s="11"/>
       <c r="E110" s="12"/>
@@ -6764,7 +6777,7 @@
       <c r="Y110" s="11"/>
       <c r="Z110" s="14"/>
     </row>
-    <row r="111" spans="2:26">
+    <row r="111" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B111" s="11"/>
       <c r="C111" s="11"/>
       <c r="E111" s="12"/>
@@ -6776,7 +6789,7 @@
       <c r="Y111" s="11"/>
       <c r="Z111" s="14"/>
     </row>
-    <row r="112" spans="2:26">
+    <row r="112" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B112" s="11"/>
       <c r="C112" s="11"/>
       <c r="E112" s="12"/>
@@ -6788,7 +6801,7 @@
       <c r="Y112" s="11"/>
       <c r="Z112" s="14"/>
     </row>
-    <row r="113" spans="2:26">
+    <row r="113" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B113" s="11"/>
       <c r="C113" s="11"/>
       <c r="E113" s="12"/>
@@ -6800,7 +6813,7 @@
       <c r="Y113" s="11"/>
       <c r="Z113" s="14"/>
     </row>
-    <row r="114" spans="2:26">
+    <row r="114" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B114" s="11"/>
       <c r="C114" s="11"/>
       <c r="E114" s="12"/>
@@ -6812,7 +6825,7 @@
       <c r="Y114" s="11"/>
       <c r="Z114" s="14"/>
     </row>
-    <row r="115" spans="2:26">
+    <row r="115" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B115" s="11"/>
       <c r="C115" s="11"/>
       <c r="E115" s="12"/>
@@ -6824,7 +6837,7 @@
       <c r="Y115" s="11"/>
       <c r="Z115" s="14"/>
     </row>
-    <row r="116" spans="2:26">
+    <row r="116" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B116" s="11"/>
       <c r="C116" s="11"/>
       <c r="E116" s="12"/>
@@ -6836,7 +6849,7 @@
       <c r="Y116" s="11"/>
       <c r="Z116" s="14"/>
     </row>
-    <row r="117" spans="2:26">
+    <row r="117" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B117" s="11"/>
       <c r="C117" s="11"/>
       <c r="E117" s="12"/>
@@ -6848,7 +6861,7 @@
       <c r="Y117" s="11"/>
       <c r="Z117" s="14"/>
     </row>
-    <row r="118" spans="2:26">
+    <row r="118" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B118" s="11"/>
       <c r="C118" s="11"/>
       <c r="E118" s="12"/>
@@ -6860,7 +6873,7 @@
       <c r="Y118" s="11"/>
       <c r="Z118" s="14"/>
     </row>
-    <row r="119" spans="2:26">
+    <row r="119" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B119" s="11"/>
       <c r="C119" s="11"/>
       <c r="E119" s="12"/>
@@ -6872,7 +6885,7 @@
       <c r="Y119" s="11"/>
       <c r="Z119" s="14"/>
     </row>
-    <row r="120" spans="2:26">
+    <row r="120" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B120" s="11"/>
       <c r="C120" s="11"/>
       <c r="E120" s="12"/>
@@ -6884,7 +6897,7 @@
       <c r="Y120" s="11"/>
       <c r="Z120" s="14"/>
     </row>
-    <row r="121" spans="2:26">
+    <row r="121" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B121" s="11"/>
       <c r="C121" s="11"/>
       <c r="E121" s="12"/>
@@ -6896,7 +6909,7 @@
       <c r="Y121" s="11"/>
       <c r="Z121" s="14"/>
     </row>
-    <row r="122" spans="2:26">
+    <row r="122" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B122" s="11"/>
       <c r="C122" s="11"/>
       <c r="E122" s="12"/>
@@ -6908,7 +6921,7 @@
       <c r="Y122" s="11"/>
       <c r="Z122" s="14"/>
     </row>
-    <row r="123" spans="2:26">
+    <row r="123" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B123" s="11"/>
       <c r="C123" s="11"/>
       <c r="E123" s="12"/>
@@ -6920,7 +6933,7 @@
       <c r="Y123" s="11"/>
       <c r="Z123" s="14"/>
     </row>
-    <row r="124" spans="2:26">
+    <row r="124" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B124" s="11"/>
       <c r="C124" s="11"/>
       <c r="E124" s="12"/>
@@ -6932,7 +6945,7 @@
       <c r="Y124" s="11"/>
       <c r="Z124" s="14"/>
     </row>
-    <row r="125" spans="2:26">
+    <row r="125" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B125" s="11"/>
       <c r="C125" s="11"/>
       <c r="E125" s="12"/>
@@ -6944,7 +6957,7 @@
       <c r="Y125" s="11"/>
       <c r="Z125" s="14"/>
     </row>
-    <row r="126" spans="2:26">
+    <row r="126" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B126" s="11"/>
       <c r="C126" s="11"/>
       <c r="E126" s="12"/>
@@ -6956,7 +6969,7 @@
       <c r="Y126" s="11"/>
       <c r="Z126" s="14"/>
     </row>
-    <row r="127" spans="2:26">
+    <row r="127" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B127" s="11"/>
       <c r="C127" s="11"/>
       <c r="E127" s="12"/>
@@ -6968,7 +6981,7 @@
       <c r="Y127" s="11"/>
       <c r="Z127" s="14"/>
     </row>
-    <row r="128" spans="2:26">
+    <row r="128" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B128" s="11"/>
       <c r="C128" s="11"/>
       <c r="E128" s="12"/>
@@ -6980,7 +6993,7 @@
       <c r="Y128" s="11"/>
       <c r="Z128" s="14"/>
     </row>
-    <row r="129" spans="2:26">
+    <row r="129" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B129" s="11"/>
       <c r="C129" s="11"/>
       <c r="E129" s="12"/>
@@ -6992,7 +7005,7 @@
       <c r="Y129" s="11"/>
       <c r="Z129" s="14"/>
     </row>
-    <row r="130" spans="2:26">
+    <row r="130" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B130" s="11"/>
       <c r="C130" s="11"/>
       <c r="E130" s="12"/>
@@ -7004,7 +7017,7 @@
       <c r="Y130" s="11"/>
       <c r="Z130" s="14"/>
     </row>
-    <row r="131" spans="2:26">
+    <row r="131" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B131" s="11"/>
       <c r="C131" s="11"/>
       <c r="E131" s="12"/>
@@ -7016,7 +7029,7 @@
       <c r="Y131" s="11"/>
       <c r="Z131" s="14"/>
     </row>
-    <row r="132" spans="2:26">
+    <row r="132" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B132" s="11"/>
       <c r="C132" s="11"/>
       <c r="E132" s="12"/>
@@ -7028,7 +7041,7 @@
       <c r="Y132" s="11"/>
       <c r="Z132" s="14"/>
     </row>
-    <row r="133" spans="2:26">
+    <row r="133" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B133" s="11"/>
       <c r="C133" s="11"/>
       <c r="E133" s="12"/>
@@ -7040,7 +7053,7 @@
       <c r="Y133" s="11"/>
       <c r="Z133" s="14"/>
     </row>
-    <row r="134" spans="2:26">
+    <row r="134" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B134" s="11"/>
       <c r="C134" s="11"/>
       <c r="E134" s="12"/>
@@ -7052,7 +7065,7 @@
       <c r="Y134" s="11"/>
       <c r="Z134" s="14"/>
     </row>
-    <row r="135" spans="2:26">
+    <row r="135" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B135" s="11"/>
       <c r="C135" s="11"/>
       <c r="E135" s="12"/>
@@ -7064,7 +7077,7 @@
       <c r="Y135" s="11"/>
       <c r="Z135" s="14"/>
     </row>
-    <row r="136" spans="2:26">
+    <row r="136" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B136" s="11"/>
       <c r="C136" s="11"/>
       <c r="E136" s="12"/>
@@ -7076,7 +7089,7 @@
       <c r="Y136" s="11"/>
       <c r="Z136" s="14"/>
     </row>
-    <row r="137" spans="2:26">
+    <row r="137" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B137" s="11"/>
       <c r="C137" s="11"/>
       <c r="E137" s="12"/>
@@ -7088,7 +7101,7 @@
       <c r="Y137" s="11"/>
       <c r="Z137" s="14"/>
     </row>
-    <row r="138" spans="2:26">
+    <row r="138" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B138" s="11"/>
       <c r="C138" s="11"/>
       <c r="E138" s="12"/>
@@ -7100,7 +7113,7 @@
       <c r="Y138" s="11"/>
       <c r="Z138" s="14"/>
     </row>
-    <row r="139" spans="2:26">
+    <row r="139" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B139" s="11"/>
       <c r="C139" s="11"/>
       <c r="E139" s="12"/>
@@ -7112,7 +7125,7 @@
       <c r="Y139" s="11"/>
       <c r="Z139" s="14"/>
     </row>
-    <row r="140" spans="2:26">
+    <row r="140" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B140" s="11"/>
       <c r="C140" s="11"/>
       <c r="E140" s="12"/>
@@ -7124,7 +7137,7 @@
       <c r="Y140" s="11"/>
       <c r="Z140" s="14"/>
     </row>
-    <row r="141" spans="2:26">
+    <row r="141" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B141" s="11"/>
       <c r="C141" s="11"/>
       <c r="E141" s="12"/>
@@ -7136,7 +7149,7 @@
       <c r="Y141" s="11"/>
       <c r="Z141" s="14"/>
     </row>
-    <row r="142" spans="2:26">
+    <row r="142" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B142" s="11"/>
       <c r="C142" s="11"/>
       <c r="E142" s="12"/>
@@ -7148,7 +7161,7 @@
       <c r="Y142" s="11"/>
       <c r="Z142" s="14"/>
     </row>
-    <row r="143" spans="2:26">
+    <row r="143" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B143" s="11"/>
       <c r="C143" s="11"/>
       <c r="E143" s="12"/>
@@ -7160,7 +7173,7 @@
       <c r="Y143" s="11"/>
       <c r="Z143" s="14"/>
     </row>
-    <row r="144" spans="2:26">
+    <row r="144" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B144" s="11"/>
       <c r="C144" s="11"/>
       <c r="E144" s="12"/>
@@ -7172,7 +7185,7 @@
       <c r="Y144" s="11"/>
       <c r="Z144" s="14"/>
     </row>
-    <row r="145" spans="2:26">
+    <row r="145" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B145" s="11"/>
       <c r="C145" s="11"/>
       <c r="E145" s="12"/>
@@ -7184,7 +7197,7 @@
       <c r="Y145" s="11"/>
       <c r="Z145" s="14"/>
     </row>
-    <row r="146" spans="2:26">
+    <row r="146" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B146" s="11"/>
       <c r="C146" s="11"/>
       <c r="E146" s="12"/>
@@ -7196,7 +7209,7 @@
       <c r="Y146" s="11"/>
       <c r="Z146" s="14"/>
     </row>
-    <row r="147" spans="2:26">
+    <row r="147" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B147" s="11"/>
       <c r="C147" s="11"/>
       <c r="E147" s="12"/>
@@ -7208,7 +7221,7 @@
       <c r="Y147" s="11"/>
       <c r="Z147" s="14"/>
     </row>
-    <row r="148" spans="2:26">
+    <row r="148" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B148" s="11"/>
       <c r="C148" s="11"/>
       <c r="E148" s="12"/>
@@ -7220,7 +7233,7 @@
       <c r="Y148" s="11"/>
       <c r="Z148" s="14"/>
     </row>
-    <row r="149" spans="2:26">
+    <row r="149" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B149" s="11"/>
       <c r="C149" s="11"/>
       <c r="E149" s="12"/>
@@ -7232,7 +7245,7 @@
       <c r="Y149" s="11"/>
       <c r="Z149" s="14"/>
     </row>
-    <row r="150" spans="2:26">
+    <row r="150" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B150" s="11"/>
       <c r="C150" s="11"/>
       <c r="E150" s="12"/>
@@ -7244,7 +7257,7 @@
       <c r="Y150" s="11"/>
       <c r="Z150" s="14"/>
     </row>
-    <row r="151" spans="2:26">
+    <row r="151" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B151" s="11"/>
       <c r="C151" s="11"/>
       <c r="E151" s="12"/>
@@ -7256,7 +7269,7 @@
       <c r="Y151" s="11"/>
       <c r="Z151" s="14"/>
     </row>
-    <row r="152" spans="2:26">
+    <row r="152" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B152" s="11"/>
       <c r="C152" s="11"/>
       <c r="E152" s="12"/>
@@ -7268,7 +7281,7 @@
       <c r="Y152" s="11"/>
       <c r="Z152" s="14"/>
     </row>
-    <row r="153" spans="2:26">
+    <row r="153" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B153" s="11"/>
       <c r="C153" s="11"/>
       <c r="E153" s="12"/>
@@ -7280,7 +7293,7 @@
       <c r="Y153" s="11"/>
       <c r="Z153" s="14"/>
     </row>
-    <row r="154" spans="2:26">
+    <row r="154" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B154" s="11"/>
       <c r="C154" s="11"/>
       <c r="E154" s="12"/>
@@ -7292,7 +7305,7 @@
       <c r="Y154" s="11"/>
       <c r="Z154" s="14"/>
     </row>
-    <row r="155" spans="2:26">
+    <row r="155" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B155" s="11"/>
       <c r="C155" s="11"/>
       <c r="E155" s="12"/>
@@ -7304,7 +7317,7 @@
       <c r="Y155" s="11"/>
       <c r="Z155" s="14"/>
     </row>
-    <row r="156" spans="2:26">
+    <row r="156" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B156" s="11"/>
       <c r="C156" s="11"/>
       <c r="E156" s="12"/>
@@ -7316,7 +7329,7 @@
       <c r="Y156" s="11"/>
       <c r="Z156" s="14"/>
     </row>
-    <row r="157" spans="2:26">
+    <row r="157" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B157" s="11"/>
       <c r="C157" s="11"/>
       <c r="E157" s="12"/>
@@ -7328,7 +7341,7 @@
       <c r="Y157" s="11"/>
       <c r="Z157" s="14"/>
     </row>
-    <row r="158" spans="2:26">
+    <row r="158" spans="2:26" x14ac:dyDescent="0.15">
       <c r="B158" s="11"/>
       <c r="C158" s="11"/>
       <c r="E158" s="12"/>
@@ -7340,604 +7353,604 @@
       <c r="Y158" s="11"/>
       <c r="Z158" s="14"/>
     </row>
-    <row r="159" spans="2:26">
+    <row r="159" spans="2:26" x14ac:dyDescent="0.15">
       <c r="X159" s="17"/>
     </row>
-    <row r="160" spans="2:26">
+    <row r="160" spans="2:26" x14ac:dyDescent="0.15">
       <c r="X160" s="17"/>
     </row>
-    <row r="161" spans="24:24">
+    <row r="161" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X161" s="17"/>
     </row>
-    <row r="162" spans="24:24">
+    <row r="162" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X162" s="17"/>
     </row>
-    <row r="163" spans="24:24">
+    <row r="163" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X163" s="17"/>
     </row>
-    <row r="164" spans="24:24">
+    <row r="164" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X164" s="17"/>
     </row>
-    <row r="165" spans="24:24">
+    <row r="165" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X165" s="17"/>
     </row>
-    <row r="166" spans="24:24">
+    <row r="166" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X166" s="17"/>
     </row>
-    <row r="167" spans="24:24">
+    <row r="167" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X167" s="17"/>
     </row>
-    <row r="168" spans="24:24">
+    <row r="168" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X168" s="17"/>
     </row>
-    <row r="169" spans="24:24">
+    <row r="169" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X169" s="17"/>
     </row>
-    <row r="170" spans="24:24">
+    <row r="170" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X170" s="17"/>
     </row>
-    <row r="171" spans="24:24">
+    <row r="171" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X171" s="17"/>
     </row>
-    <row r="172" spans="24:24">
+    <row r="172" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X172" s="17"/>
     </row>
-    <row r="173" spans="24:24">
+    <row r="173" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X173" s="17"/>
     </row>
-    <row r="174" spans="24:24">
+    <row r="174" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X174" s="17"/>
     </row>
-    <row r="175" spans="24:24">
+    <row r="175" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X175" s="17"/>
     </row>
-    <row r="176" spans="24:24">
+    <row r="176" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X176" s="17"/>
     </row>
-    <row r="177" spans="24:24">
+    <row r="177" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X177" s="17"/>
     </row>
-    <row r="178" spans="24:24">
+    <row r="178" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X178" s="17"/>
     </row>
-    <row r="179" spans="24:24">
+    <row r="179" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X179" s="17"/>
     </row>
-    <row r="180" spans="24:24">
+    <row r="180" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X180" s="17"/>
     </row>
-    <row r="181" spans="24:24">
+    <row r="181" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X181" s="17"/>
     </row>
-    <row r="182" spans="24:24">
+    <row r="182" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X182" s="17"/>
     </row>
-    <row r="183" spans="24:24">
+    <row r="183" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X183" s="17"/>
     </row>
-    <row r="184" spans="24:24">
+    <row r="184" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X184" s="17"/>
     </row>
-    <row r="185" spans="24:24">
+    <row r="185" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X185" s="17"/>
     </row>
-    <row r="186" spans="24:24">
+    <row r="186" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X186" s="17"/>
     </row>
-    <row r="187" spans="24:24">
+    <row r="187" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X187" s="17"/>
     </row>
-    <row r="188" spans="24:24">
+    <row r="188" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X188" s="17"/>
     </row>
-    <row r="189" spans="24:24">
+    <row r="189" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X189" s="17"/>
     </row>
-    <row r="190" spans="24:24">
+    <row r="190" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X190" s="17"/>
     </row>
-    <row r="191" spans="24:24">
+    <row r="191" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X191" s="17"/>
     </row>
-    <row r="192" spans="24:24">
+    <row r="192" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X192" s="17"/>
     </row>
-    <row r="193" spans="24:24">
+    <row r="193" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X193" s="17"/>
     </row>
-    <row r="194" spans="24:24">
+    <row r="194" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X194" s="17"/>
     </row>
-    <row r="195" spans="24:24">
+    <row r="195" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X195" s="17"/>
     </row>
-    <row r="196" spans="24:24">
+    <row r="196" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X196" s="17"/>
     </row>
-    <row r="197" spans="24:24">
+    <row r="197" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X197" s="17"/>
     </row>
-    <row r="198" spans="24:24">
+    <row r="198" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X198" s="17"/>
     </row>
-    <row r="199" spans="24:24">
+    <row r="199" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X199" s="17"/>
     </row>
-    <row r="200" spans="24:24">
+    <row r="200" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X200" s="17"/>
     </row>
-    <row r="201" spans="24:24">
+    <row r="201" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X201" s="17"/>
     </row>
-    <row r="202" spans="24:24">
+    <row r="202" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X202" s="17"/>
     </row>
-    <row r="203" spans="24:24">
+    <row r="203" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X203" s="17"/>
     </row>
-    <row r="204" spans="24:24">
+    <row r="204" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X204" s="17"/>
     </row>
-    <row r="205" spans="24:24">
+    <row r="205" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X205" s="17"/>
     </row>
-    <row r="206" spans="24:24">
+    <row r="206" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X206" s="17"/>
     </row>
-    <row r="207" spans="24:24">
+    <row r="207" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X207" s="17"/>
     </row>
-    <row r="208" spans="24:24">
+    <row r="208" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X208" s="17"/>
     </row>
-    <row r="209" spans="24:24">
+    <row r="209" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X209" s="17"/>
     </row>
-    <row r="210" spans="24:24">
+    <row r="210" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X210" s="17"/>
     </row>
-    <row r="211" spans="24:24">
+    <row r="211" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X211" s="17"/>
     </row>
-    <row r="212" spans="24:24">
+    <row r="212" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X212" s="17"/>
     </row>
-    <row r="213" spans="24:24">
+    <row r="213" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X213" s="17"/>
     </row>
-    <row r="214" spans="24:24">
+    <row r="214" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X214" s="17"/>
     </row>
-    <row r="215" spans="24:24">
+    <row r="215" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X215" s="17"/>
     </row>
-    <row r="216" spans="24:24">
+    <row r="216" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X216" s="17"/>
     </row>
-    <row r="217" spans="24:24">
+    <row r="217" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X217" s="17"/>
     </row>
-    <row r="218" spans="24:24">
+    <row r="218" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X218" s="17"/>
     </row>
-    <row r="219" spans="24:24">
+    <row r="219" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X219" s="17"/>
     </row>
-    <row r="220" spans="24:24">
+    <row r="220" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X220" s="17"/>
     </row>
-    <row r="221" spans="24:24">
+    <row r="221" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X221" s="17"/>
     </row>
-    <row r="222" spans="24:24">
+    <row r="222" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X222" s="17"/>
     </row>
-    <row r="223" spans="24:24">
+    <row r="223" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X223" s="17"/>
     </row>
-    <row r="224" spans="24:24">
+    <row r="224" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X224" s="17"/>
     </row>
-    <row r="225" spans="24:24">
+    <row r="225" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X225" s="17"/>
     </row>
-    <row r="226" spans="24:24">
+    <row r="226" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X226" s="17"/>
     </row>
-    <row r="227" spans="24:24">
+    <row r="227" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X227" s="17"/>
     </row>
-    <row r="228" spans="24:24">
+    <row r="228" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X228" s="17"/>
     </row>
-    <row r="229" spans="24:24">
+    <row r="229" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X229" s="17"/>
     </row>
-    <row r="230" spans="24:24">
+    <row r="230" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X230" s="17"/>
     </row>
-    <row r="231" spans="24:24">
+    <row r="231" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X231" s="17"/>
     </row>
-    <row r="232" spans="24:24">
+    <row r="232" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X232" s="17"/>
     </row>
-    <row r="233" spans="24:24">
+    <row r="233" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X233" s="17"/>
     </row>
-    <row r="234" spans="24:24">
+    <row r="234" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X234" s="17"/>
     </row>
-    <row r="235" spans="24:24">
+    <row r="235" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X235" s="17"/>
     </row>
-    <row r="236" spans="24:24">
+    <row r="236" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X236" s="17"/>
     </row>
-    <row r="237" spans="24:24">
+    <row r="237" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X237" s="17"/>
     </row>
-    <row r="238" spans="24:24">
+    <row r="238" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X238" s="17"/>
     </row>
-    <row r="239" spans="24:24">
+    <row r="239" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X239" s="17"/>
     </row>
-    <row r="240" spans="24:24">
+    <row r="240" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X240" s="17"/>
     </row>
-    <row r="241" spans="24:24">
+    <row r="241" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X241" s="17"/>
     </row>
-    <row r="242" spans="24:24">
+    <row r="242" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X242" s="17"/>
     </row>
-    <row r="243" spans="24:24">
+    <row r="243" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X243" s="17"/>
     </row>
-    <row r="244" spans="24:24">
+    <row r="244" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X244" s="17"/>
     </row>
-    <row r="245" spans="24:24">
+    <row r="245" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X245" s="17"/>
     </row>
-    <row r="246" spans="24:24">
+    <row r="246" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X246" s="17"/>
     </row>
-    <row r="247" spans="24:24">
+    <row r="247" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X247" s="17"/>
     </row>
-    <row r="248" spans="24:24">
+    <row r="248" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X248" s="17"/>
     </row>
-    <row r="249" spans="24:24">
+    <row r="249" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X249" s="17"/>
     </row>
-    <row r="250" spans="24:24">
+    <row r="250" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X250" s="17"/>
     </row>
-    <row r="251" spans="24:24">
+    <row r="251" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X251" s="17"/>
     </row>
-    <row r="252" spans="24:24">
+    <row r="252" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X252" s="17"/>
     </row>
-    <row r="253" spans="24:24">
+    <row r="253" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X253" s="17"/>
     </row>
-    <row r="254" spans="24:24">
+    <row r="254" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X254" s="17"/>
     </row>
-    <row r="255" spans="24:24">
+    <row r="255" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X255" s="17"/>
     </row>
-    <row r="256" spans="24:24">
+    <row r="256" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X256" s="17"/>
     </row>
-    <row r="257" spans="24:24">
+    <row r="257" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X257" s="17"/>
     </row>
-    <row r="258" spans="24:24">
+    <row r="258" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X258" s="17"/>
     </row>
-    <row r="259" spans="24:24">
+    <row r="259" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X259" s="17"/>
     </row>
-    <row r="260" spans="24:24">
+    <row r="260" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X260" s="17"/>
     </row>
-    <row r="261" spans="24:24">
+    <row r="261" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X261" s="17"/>
     </row>
-    <row r="262" spans="24:24">
+    <row r="262" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X262" s="17"/>
     </row>
-    <row r="263" spans="24:24">
+    <row r="263" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X263" s="17"/>
     </row>
-    <row r="264" spans="24:24">
+    <row r="264" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X264" s="17"/>
     </row>
-    <row r="265" spans="24:24">
+    <row r="265" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X265" s="17"/>
     </row>
-    <row r="266" spans="24:24">
+    <row r="266" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X266" s="17"/>
     </row>
-    <row r="267" spans="24:24">
+    <row r="267" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X267" s="17"/>
     </row>
-    <row r="268" spans="24:24">
+    <row r="268" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X268" s="17"/>
     </row>
-    <row r="269" spans="24:24">
+    <row r="269" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X269" s="17"/>
     </row>
-    <row r="270" spans="24:24">
+    <row r="270" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X270" s="17"/>
     </row>
-    <row r="271" spans="24:24">
+    <row r="271" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X271" s="17"/>
     </row>
-    <row r="272" spans="24:24">
+    <row r="272" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X272" s="17"/>
     </row>
-    <row r="273" spans="24:24">
+    <row r="273" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X273" s="17"/>
     </row>
-    <row r="274" spans="24:24">
+    <row r="274" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X274" s="17"/>
     </row>
-    <row r="275" spans="24:24">
+    <row r="275" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X275" s="17"/>
     </row>
-    <row r="276" spans="24:24">
+    <row r="276" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X276" s="17"/>
     </row>
-    <row r="277" spans="24:24">
+    <row r="277" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X277" s="17"/>
     </row>
-    <row r="278" spans="24:24">
+    <row r="278" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X278" s="17"/>
     </row>
-    <row r="279" spans="24:24">
+    <row r="279" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X279" s="17"/>
     </row>
-    <row r="280" spans="24:24">
+    <row r="280" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X280" s="17"/>
     </row>
-    <row r="281" spans="24:24">
+    <row r="281" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X281" s="17"/>
     </row>
-    <row r="282" spans="24:24">
+    <row r="282" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X282" s="17"/>
     </row>
-    <row r="283" spans="24:24">
+    <row r="283" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X283" s="17"/>
     </row>
-    <row r="284" spans="24:24">
+    <row r="284" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X284" s="17"/>
     </row>
-    <row r="285" spans="24:24">
+    <row r="285" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X285" s="17"/>
     </row>
-    <row r="286" spans="24:24">
+    <row r="286" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X286" s="17"/>
     </row>
-    <row r="287" spans="24:24">
+    <row r="287" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X287" s="17"/>
     </row>
-    <row r="288" spans="24:24">
+    <row r="288" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X288" s="17"/>
     </row>
-    <row r="289" spans="24:24">
+    <row r="289" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X289" s="17"/>
     </row>
-    <row r="290" spans="24:24">
+    <row r="290" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X290" s="17"/>
     </row>
-    <row r="291" spans="24:24">
+    <row r="291" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X291" s="17"/>
     </row>
-    <row r="292" spans="24:24">
+    <row r="292" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X292" s="17"/>
     </row>
-    <row r="293" spans="24:24">
+    <row r="293" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X293" s="17"/>
     </row>
-    <row r="294" spans="24:24">
+    <row r="294" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X294" s="17"/>
     </row>
-    <row r="295" spans="24:24">
+    <row r="295" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X295" s="17"/>
     </row>
-    <row r="296" spans="24:24">
+    <row r="296" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X296" s="17"/>
     </row>
-    <row r="297" spans="24:24">
+    <row r="297" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X297" s="17"/>
     </row>
-    <row r="298" spans="24:24">
+    <row r="298" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X298" s="17"/>
     </row>
-    <row r="299" spans="24:24">
+    <row r="299" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X299" s="17"/>
     </row>
-    <row r="300" spans="24:24">
+    <row r="300" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X300" s="17"/>
     </row>
-    <row r="301" spans="24:24">
+    <row r="301" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X301" s="17"/>
     </row>
-    <row r="302" spans="24:24">
+    <row r="302" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X302" s="17"/>
     </row>
-    <row r="303" spans="24:24">
+    <row r="303" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X303" s="17"/>
     </row>
-    <row r="304" spans="24:24">
+    <row r="304" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X304" s="17"/>
     </row>
-    <row r="305" spans="24:24">
+    <row r="305" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X305" s="17"/>
     </row>
-    <row r="306" spans="24:24">
+    <row r="306" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X306" s="17"/>
     </row>
-    <row r="307" spans="24:24">
+    <row r="307" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X307" s="17"/>
     </row>
-    <row r="308" spans="24:24">
+    <row r="308" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X308" s="17"/>
     </row>
-    <row r="309" spans="24:24">
+    <row r="309" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X309" s="17"/>
     </row>
-    <row r="310" spans="24:24">
+    <row r="310" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X310" s="17"/>
     </row>
-    <row r="311" spans="24:24">
+    <row r="311" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X311" s="17"/>
     </row>
-    <row r="312" spans="24:24">
+    <row r="312" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X312" s="17"/>
     </row>
-    <row r="313" spans="24:24">
+    <row r="313" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X313" s="17"/>
     </row>
-    <row r="314" spans="24:24">
+    <row r="314" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X314" s="17"/>
     </row>
-    <row r="315" spans="24:24">
+    <row r="315" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X315" s="17"/>
     </row>
-    <row r="316" spans="24:24">
+    <row r="316" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X316" s="17"/>
     </row>
-    <row r="317" spans="24:24">
+    <row r="317" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X317" s="17"/>
     </row>
-    <row r="318" spans="24:24">
+    <row r="318" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X318" s="17"/>
     </row>
-    <row r="319" spans="24:24">
+    <row r="319" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X319" s="17"/>
     </row>
-    <row r="320" spans="24:24">
+    <row r="320" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X320" s="17"/>
     </row>
-    <row r="321" spans="24:24">
+    <row r="321" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X321" s="17"/>
     </row>
-    <row r="322" spans="24:24">
+    <row r="322" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X322" s="17"/>
     </row>
-    <row r="323" spans="24:24">
+    <row r="323" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X323" s="17"/>
     </row>
-    <row r="324" spans="24:24">
+    <row r="324" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X324" s="17"/>
     </row>
-    <row r="325" spans="24:24">
+    <row r="325" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X325" s="17"/>
     </row>
-    <row r="326" spans="24:24">
+    <row r="326" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X326" s="17"/>
     </row>
-    <row r="327" spans="24:24">
+    <row r="327" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X327" s="17"/>
     </row>
-    <row r="328" spans="24:24">
+    <row r="328" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X328" s="17"/>
     </row>
-    <row r="329" spans="24:24">
+    <row r="329" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X329" s="17"/>
     </row>
-    <row r="330" spans="24:24">
+    <row r="330" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X330" s="17"/>
     </row>
-    <row r="331" spans="24:24">
+    <row r="331" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X331" s="17"/>
     </row>
-    <row r="332" spans="24:24">
+    <row r="332" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X332" s="17"/>
     </row>
-    <row r="333" spans="24:24">
+    <row r="333" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X333" s="17"/>
     </row>
-    <row r="334" spans="24:24">
+    <row r="334" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X334" s="17"/>
     </row>
-    <row r="335" spans="24:24">
+    <row r="335" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X335" s="17"/>
     </row>
-    <row r="336" spans="24:24">
+    <row r="336" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X336" s="17"/>
     </row>
-    <row r="337" spans="24:24">
+    <row r="337" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X337" s="17"/>
     </row>
-    <row r="338" spans="24:24">
+    <row r="338" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X338" s="17"/>
     </row>
-    <row r="339" spans="24:24">
+    <row r="339" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X339" s="17"/>
     </row>
-    <row r="340" spans="24:24">
+    <row r="340" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X340" s="17"/>
     </row>
-    <row r="341" spans="24:24">
+    <row r="341" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X341" s="17"/>
     </row>
-    <row r="342" spans="24:24">
+    <row r="342" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X342" s="17"/>
     </row>
-    <row r="343" spans="24:24">
+    <row r="343" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X343" s="17"/>
     </row>
-    <row r="344" spans="24:24">
+    <row r="344" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X344" s="17"/>
     </row>
-    <row r="345" spans="24:24">
+    <row r="345" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X345" s="17"/>
     </row>
-    <row r="346" spans="24:24">
+    <row r="346" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X346" s="17"/>
     </row>
-    <row r="347" spans="24:24">
+    <row r="347" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X347" s="17"/>
     </row>
-    <row r="348" spans="24:24">
+    <row r="348" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X348" s="17"/>
     </row>
-    <row r="349" spans="24:24">
+    <row r="349" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X349" s="17"/>
     </row>
-    <row r="350" spans="24:24">
+    <row r="350" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X350" s="17"/>
     </row>
-    <row r="351" spans="24:24">
+    <row r="351" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X351" s="17"/>
     </row>
-    <row r="352" spans="24:24">
+    <row r="352" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X352" s="17"/>
     </row>
-    <row r="353" spans="24:24">
+    <row r="353" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X353" s="17"/>
     </row>
-    <row r="354" spans="24:24">
+    <row r="354" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X354" s="17"/>
     </row>
-    <row r="355" spans="24:24">
+    <row r="355" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X355" s="17"/>
     </row>
-    <row r="356" spans="24:24">
+    <row r="356" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X356" s="17"/>
     </row>
-    <row r="357" spans="24:24">
+    <row r="357" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X357" s="17"/>
     </row>
-    <row r="358" spans="24:24">
+    <row r="358" spans="24:24" x14ac:dyDescent="0.15">
       <c r="X358" s="17"/>
     </row>
   </sheetData>
@@ -7988,7 +8001,7 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75" customHeight="1" zeroHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15.75" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="9" style="60"/>
   </cols>
@@ -8002,20 +8015,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62760D14-1F64-4D73-BBAC-22718A84BD18}">
   <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="11.65"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="2.46484375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30.1328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="15.6640625" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.796875" style="1"/>
+    <col min="6" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B1" s="20" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A2" s="31"/>
       <c r="B2" s="32" t="s">
         <v>14</v>
@@ -8024,7 +8037,7 @@
       <c r="D2" s="22"/>
       <c r="E2" s="18"/>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C3" s="28" t="s">
         <v>15</v>
       </c>
@@ -8035,22 +8048,22 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B4" s="33" t="s">
         <v>18</v>
       </c>
       <c r="C4" s="34">
-        <v>4.2699999999999995E-2</v>
+        <v>4.2900000000000001E-2</v>
       </c>
       <c r="D4" s="34">
         <v>7.4999999999999997E-2</v>
       </c>
       <c r="E4" s="35">
         <f>D4-C4</f>
-        <v>3.2300000000000002E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+        <v>3.2099999999999997E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B5" s="33" t="s">
         <v>19</v>
       </c>
@@ -8065,7 +8078,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B6" s="33" t="s">
         <v>20</v>
       </c>
@@ -8080,13 +8093,13 @@
         <v>1.7999999999999995E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A8" s="31"/>
       <c r="B8" s="32" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B9" s="1" t="s">
         <v>52</v>
       </c>
@@ -8094,7 +8107,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B10" s="26" t="s">
         <v>23</v>
       </c>
@@ -8102,7 +8115,7 @@
         <v>9.9400000000000002E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B11" s="26" t="s">
         <v>24</v>
       </c>
@@ -8110,7 +8123,7 @@
         <v>0.1174</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B12" s="26" t="s">
         <v>25</v>
       </c>
@@ -8118,7 +8131,7 @@
         <v>3.4500000000000003E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B13" s="26" t="s">
         <v>26</v>
       </c>
@@ -8126,7 +8139,7 @@
         <v>3.3099999999999997E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B14" s="26" t="s">
         <v>27</v>
       </c>
@@ -8134,7 +8147,7 @@
         <v>4.2299999999999997E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B15" s="26" t="s">
         <v>28</v>
       </c>
@@ -8142,7 +8155,7 @@
         <v>5.1200000000000002E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B16" s="36" t="s">
         <v>59</v>
       </c>
@@ -8154,7 +8167,7 @@
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A18" s="31"/>
       <c r="B18" s="32" t="s">
         <v>29</v>
@@ -8163,7 +8176,7 @@
       <c r="D18" s="22"/>
       <c r="E18" s="18"/>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B19" s="18" t="s">
         <v>30</v>
       </c>
@@ -8171,7 +8184,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B20" s="1" t="s">
         <v>32</v>
       </c>
@@ -8179,7 +8192,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B21" s="1" t="s">
         <v>34</v>
       </c>
@@ -8187,10 +8200,10 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C22" s="38"/>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B23" s="1" t="s">
         <v>36</v>
       </c>
@@ -8198,7 +8211,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B24" s="1" t="s">
         <v>38</v>
       </c>
@@ -8206,10 +8219,10 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C25" s="38"/>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B26" s="1" t="s">
         <v>40</v>
       </c>
@@ -8217,7 +8230,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B27" s="1" t="s">
         <v>42</v>
       </c>
@@ -8225,10 +8238,10 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="C28" s="38"/>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B29" s="1" t="s">
         <v>44</v>
       </c>
@@ -8236,7 +8249,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.15">
       <c r="B31" s="1" t="s">
         <v>46</v>
       </c>
@@ -8265,24 +8278,24 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D81F047E-EC38-4C3A-BA81-E6C9549453D6}">
   <dimension ref="A1:L29"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="2.6640625" style="53" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="53" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.796875" style="53" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" style="53" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" style="53"/>
     <col min="5" max="6" width="15.6640625" style="53" customWidth="1"/>
     <col min="7" max="8" width="10" style="53" customWidth="1"/>
     <col min="9" max="16384" width="9" style="53"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="13.15">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A1" s="51"/>
       <c r="B1" s="52" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="29.75" customHeight="1">
+    <row r="2" spans="1:12" ht="29.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B2" s="54" t="s">
         <v>2</v>
       </c>
@@ -8317,7 +8330,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B3" s="65" t="s">
         <v>26</v>
       </c>
@@ -8335,7 +8348,7 @@
       </c>
       <c r="G3" s="61">
         <f>F3/$F$10</f>
-        <v>0.53308247099404205</v>
+        <v>0.53450715296337059</v>
       </c>
       <c r="H3" s="78">
         <f>Portfolio_Mgmt!E66</f>
@@ -8354,13 +8367,13 @@
         <v>189</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B4" s="66" t="s">
         <v>328</v>
       </c>
       <c r="C4" s="63">
         <f>VLOOKUP(B4,Opportunities!B$3:E$30,3,FALSE)</f>
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="D4" s="62" t="str">
         <f>VLOOKUP(B4,Opportunities!B$3:E$30,4,FALSE)</f>
@@ -8371,11 +8384,11 @@
       </c>
       <c r="F4" s="64">
         <f>E4*C4</f>
-        <v>68400</v>
+        <v>68100</v>
       </c>
       <c r="G4" s="61">
         <f>F4/$F$10</f>
-        <v>0.21448730009407338</v>
+        <v>0.21411727715767961</v>
       </c>
       <c r="H4" s="61">
         <f>VLOOKUP(B4,Opportunities!B$3:I$30,8,FALSE)</f>
@@ -8398,13 +8411,13 @@
         <v>18.773924722806626</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B5" s="66" t="s">
         <v>329</v>
       </c>
       <c r="C5" s="63">
         <f>VLOOKUP(B5,Opportunities!B$3:E$30,3,FALSE)</f>
-        <v>16.100000000000001</v>
+        <v>15.99</v>
       </c>
       <c r="D5" s="62" t="str">
         <f>VLOOKUP(B5,Opportunities!B$3:E$30,4,FALSE)</f>
@@ -8415,11 +8428,11 @@
       </c>
       <c r="F5" s="64">
         <f>C5*E5</f>
-        <v>80500</v>
+        <v>79950</v>
       </c>
       <c r="G5" s="61">
         <f>F5/$F$10</f>
-        <v>0.2524302289118846</v>
+        <v>0.25137556987894988</v>
       </c>
       <c r="H5" s="61">
         <f>VLOOKUP(B5,Opportunities!B$3:I$30,8,FALSE)</f>
@@ -8442,7 +8455,7 @@
         <v>16.202875796143875</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B6" s="66"/>
       <c r="C6" s="63"/>
       <c r="D6" s="62"/>
@@ -8455,7 +8468,7 @@
       <c r="K6" s="84"/>
       <c r="L6" s="84"/>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B7" s="66"/>
       <c r="C7" s="63"/>
       <c r="D7" s="62"/>
@@ -8468,7 +8481,7 @@
       <c r="K7" s="84"/>
       <c r="L7" s="84"/>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B8" s="66"/>
       <c r="C8" s="63"/>
       <c r="D8" s="62"/>
@@ -8481,13 +8494,13 @@
       <c r="K8" s="84"/>
       <c r="L8" s="84"/>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B9" s="55"/>
       <c r="C9" s="58"/>
       <c r="D9" s="55"/>
       <c r="H9" s="77"/>
     </row>
-    <row r="10" spans="1:12" ht="13.15">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B10" s="67"/>
       <c r="C10" s="68"/>
       <c r="D10" s="67"/>
@@ -8496,7 +8509,7 @@
       </c>
       <c r="F10" s="69">
         <f>SUM(F3:F8)</f>
-        <v>318900</v>
+        <v>318050</v>
       </c>
       <c r="G10" s="70">
         <f>SUM(G3:G8)</f>
@@ -8519,20 +8532,20 @@
         <v>189</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B11" s="55"/>
       <c r="C11" s="58"/>
       <c r="D11" s="55"/>
       <c r="E11" s="59"/>
       <c r="F11" s="59"/>
     </row>
-    <row r="12" spans="1:12" ht="13.15">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A12" s="51"/>
       <c r="B12" s="52" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B13" s="66"/>
       <c r="C13" s="63"/>
       <c r="D13" s="62"/>
@@ -8545,7 +8558,7 @@
       <c r="K13" s="84"/>
       <c r="L13" s="84"/>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B14" s="66"/>
       <c r="C14" s="63"/>
       <c r="D14" s="62"/>
@@ -8558,7 +8571,7 @@
       <c r="K14" s="84"/>
       <c r="L14" s="84"/>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B15" s="66"/>
       <c r="C15" s="63"/>
       <c r="D15" s="62"/>
@@ -8571,7 +8584,7 @@
       <c r="K15" s="84"/>
       <c r="L15" s="84"/>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.15">
       <c r="B16" s="66"/>
       <c r="C16" s="63"/>
       <c r="D16" s="62"/>
@@ -8584,11 +8597,11 @@
       <c r="K16" s="84"/>
       <c r="L16" s="84"/>
     </row>
-    <row r="17" spans="2:12">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.15">
       <c r="G17" s="75"/>
       <c r="H17" s="75"/>
     </row>
-    <row r="18" spans="2:12" ht="13.15">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.15">
       <c r="B18" s="71" t="s">
         <v>159</v>
       </c>
@@ -8608,7 +8621,7 @@
       </c>
       <c r="G18" s="76">
         <f t="shared" ref="G18" si="0">F18/$F$10</f>
-        <v>0.53308247099404205</v>
+        <v>0.53450715296337059</v>
       </c>
       <c r="H18" s="76">
         <f>Portfolio_Mgmt!E66</f>
@@ -8627,42 +8640,42 @@
         <v>189</v>
       </c>
     </row>
-    <row r="24" spans="2:12">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.15">
       <c r="B24" s="55"/>
       <c r="C24" s="58"/>
       <c r="D24" s="55"/>
       <c r="E24" s="59"/>
       <c r="F24" s="59"/>
     </row>
-    <row r="25" spans="2:12">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.15">
       <c r="B25" s="55"/>
       <c r="C25" s="58"/>
       <c r="D25" s="55"/>
       <c r="E25" s="59"/>
       <c r="F25" s="59"/>
     </row>
-    <row r="26" spans="2:12">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.15">
       <c r="B26" s="55"/>
       <c r="C26" s="58"/>
       <c r="D26" s="55"/>
       <c r="E26" s="59"/>
       <c r="F26" s="59"/>
     </row>
-    <row r="27" spans="2:12">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.15">
       <c r="B27" s="55"/>
       <c r="C27" s="58"/>
       <c r="D27" s="55"/>
       <c r="E27" s="59"/>
       <c r="F27" s="59"/>
     </row>
-    <row r="28" spans="2:12">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.15">
       <c r="B28" s="55"/>
       <c r="C28" s="58"/>
       <c r="D28" s="55"/>
       <c r="E28" s="59"/>
       <c r="F28" s="59"/>
     </row>
-    <row r="29" spans="2:12">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.15">
       <c r="B29" s="55"/>
       <c r="C29" s="56"/>
       <c r="D29" s="55"/>
@@ -8679,78 +8692,78 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE447BDC-FAEF-412F-B13E-867203D1820E}">
   <dimension ref="A1:D41"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.65"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="2.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="27.1328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.1640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="34.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="28.796875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" style="1" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B1" s="20" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="5"/>
       <c r="B2" s="6" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B3" s="126" t="s">
         <v>88</v>
       </c>
       <c r="C3" s="126"/>
       <c r="D3" s="126"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B5" s="127" t="s">
         <v>90</v>
       </c>
       <c r="C5" s="128"/>
       <c r="D5" s="128"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B6" s="127" t="s">
         <v>91</v>
       </c>
       <c r="C6" s="128"/>
       <c r="D6" s="128"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B8" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A10" s="5"/>
       <c r="B10" s="6" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B11" s="126" t="s">
         <v>93</v>
       </c>
       <c r="C11" s="126"/>
       <c r="D11" s="126"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B12" s="126" t="s">
         <v>94</v>
       </c>
       <c r="C12" s="126"/>
       <c r="D12" s="126"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B14" s="23" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="12.4">
+    <row r="16" spans="1:4" ht="14" x14ac:dyDescent="0.2">
       <c r="B16" s="30" t="s">
         <v>103</v>
       </c>
@@ -8758,7 +8771,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B17" s="26" t="s">
         <v>95</v>
       </c>
@@ -8766,7 +8779,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B18" s="26" t="s">
         <v>96</v>
       </c>
@@ -8774,7 +8787,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B19" s="26" t="s">
         <v>97</v>
       </c>
@@ -8782,7 +8795,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B20" s="26" t="s">
         <v>98</v>
       </c>
@@ -8790,7 +8803,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B21" s="26" t="s">
         <v>118</v>
       </c>
@@ -8798,7 +8811,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B22" s="26" t="s">
         <v>120</v>
       </c>
@@ -8806,7 +8819,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B23" s="26" t="s">
         <v>122</v>
       </c>
@@ -8814,7 +8827,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B24" s="26" t="s">
         <v>127</v>
       </c>
@@ -8822,7 +8835,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B25" s="26" t="s">
         <v>124</v>
       </c>
@@ -8830,33 +8843,33 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A27" s="5"/>
       <c r="B27" s="6" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B28" s="126" t="s">
         <v>106</v>
       </c>
       <c r="C28" s="126"/>
       <c r="D28" s="126"/>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.15">
       <c r="B29" s="126" t="s">
         <v>107</v>
       </c>
       <c r="C29" s="126"/>
       <c r="D29" s="126"/>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A31" s="5"/>
       <c r="B31" s="6" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A32" s="28" t="s">
         <v>60</v>
       </c>
@@ -8864,12 +8877,12 @@
         <v>109</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.15">
       <c r="B33" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A35" s="28" t="s">
         <v>112</v>
       </c>
@@ -8877,28 +8890,28 @@
         <v>111</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.15">
       <c r="B36" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A38" s="5"/>
       <c r="B38" s="6" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.15">
       <c r="B39" s="24" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.15">
       <c r="B40" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.15">
       <c r="B41" s="1" t="s">
         <v>117</v>
       </c>

</xml_diff>